<commit_message>
Model rebuild: 3 rev streams, 3 GMs, AI deferred mechanic, aggressive RFC buyback+SBC
</commit_message>
<xml_diff>
--- a/WDAY_Model.xlsx
+++ b/WDAY_Model.xlsx
@@ -20,6 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sens_SBC" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sens_Growth" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sens_Pricing" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue_Build" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AI_Deferred" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -28,7 +30,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
@@ -37,6 +39,7 @@
     <numFmt numFmtId="169" formatCode="#,##0.0"/>
     <numFmt numFmtId="170" formatCode="&quot;$&quot;#,##0.00"/>
     <numFmt numFmtId="171" formatCode="&quot;$&quot;#,##0"/>
+    <numFmt numFmtId="172" formatCode="+#,##0;-#,##0"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -136,7 +139,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,6 +171,7 @@
     <xf numFmtId="171" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -689,7 +693,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>+77.2%</t>
+          <t>+115.4%</t>
         </is>
       </c>
     </row>
@@ -701,7 +705,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>+104.9%</t>
+          <t>+152.9%</t>
         </is>
       </c>
     </row>
@@ -754,17 +758,17 @@
         <v>0.35</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>468.37</v>
+        <v>592.42</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>2.621</v>
+        <v>3.58</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>0.536</v>
+        <v>0.6609999999999999</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>22x FCF on $21.15 FY29 FCF/share growing 18% = $468 + $17 cum cap return = TSR +262%</t>
+          <t>28x FCF on $21.39 FY29 FCF/share growing 20% = $592 + $22 cum cap return = TSR +358%</t>
         </is>
       </c>
     </row>
@@ -778,17 +782,17 @@
         <v>0.35</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>111.25</v>
+        <v>125.57</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>-0.062</v>
+        <v>0.063</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>-0.021</v>
+        <v>0.021</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>9x FCF on $11.11 FY29 FCF/share growing -10% = $111 + $32 cum cap return = TSR -6%</t>
+          <t>9x FCF on $13.84 FY29 FCF/share growing -8% = $126 + $38 cum cap return = TSR +6%</t>
         </is>
       </c>
     </row>
@@ -802,17 +806,17 @@
         <v>0.3</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>72.90000000000001</v>
+        <v>73.65000000000001</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>-0.412</v>
+        <v>-0.405</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>-0.162</v>
+        <v>-0.159</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>7x FCF on $7.81 FY29 FCF/share growing -10% = $73 + $15 cum cap return = TSR -41%</t>
+          <t>7x FCF on $8.03 FY29 FCF/share growing -10% = $74 + $15 cum cap return = TSR -40%</t>
         </is>
       </c>
     </row>
@@ -934,28 +938,28 @@
         <v>0</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.075</v>
+        <v>0.065</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>0.045</v>
+        <v>0.039</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0.03</v>
+        <v>0.026</v>
       </c>
       <c r="G6" s="21" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="16" t="n">
-        <v>10158</v>
+        <v>9981</v>
       </c>
       <c r="I6" s="16" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="16" t="n">
-        <v>662</v>
+        <v>574</v>
       </c>
     </row>
     <row r="7">
@@ -968,28 +972,28 @@
         <v>0.08</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>0.17</v>
+        <v>0.14</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>0.045</v>
+        <v>0.03</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>0.027</v>
+        <v>0.018</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>0.018</v>
+        <v>0.012</v>
       </c>
       <c r="G7" s="21" t="n">
         <v>0.08</v>
       </c>
       <c r="H7" s="16" t="n">
-        <v>11885</v>
+        <v>11379</v>
       </c>
       <c r="I7" s="16" t="n">
-        <v>813</v>
+        <v>799</v>
       </c>
       <c r="J7" s="16" t="n">
-        <v>457</v>
+        <v>299</v>
       </c>
     </row>
     <row r="8">
@@ -1002,28 +1006,28 @@
         <v>0.18</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.04</v>
+        <v>0.025</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>0.024</v>
+        <v>0.015</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>0.016</v>
+        <v>0.01</v>
       </c>
       <c r="G8" s="21" t="n">
         <v>0.1</v>
       </c>
       <c r="H8" s="16" t="n">
-        <v>14024</v>
+        <v>13085</v>
       </c>
       <c r="I8" s="16" t="n">
-        <v>1188</v>
+        <v>1138</v>
       </c>
       <c r="J8" s="16" t="n">
-        <v>475</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9">
@@ -1036,28 +1040,28 @@
         <v>0.3</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>0.02</v>
+        <v>0.005</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>0.012</v>
+        <v>0.003</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>0.008</v>
+        <v>0.002</v>
       </c>
       <c r="G9" s="21" t="n">
         <v>0.12</v>
       </c>
       <c r="H9" s="16" t="n">
-        <v>16268</v>
+        <v>14787</v>
       </c>
       <c r="I9" s="16" t="n">
-        <v>1683</v>
+        <v>1570</v>
       </c>
       <c r="J9" s="16" t="n">
-        <v>280</v>
+        <v>65</v>
       </c>
     </row>
     <row r="11">
@@ -1138,28 +1142,28 @@
         <v>0</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>-0.05</v>
+        <v>0.05</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>-0.025</v>
+        <v>0.025</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>-0.015</v>
+        <v>0.015</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>-0.01</v>
+        <v>0.01</v>
       </c>
       <c r="G13" s="21" t="n">
         <v>0</v>
       </c>
       <c r="H13" s="16" t="n">
-        <v>8391</v>
+        <v>9275</v>
       </c>
       <c r="I13" s="16" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="16" t="n">
-        <v>-221</v>
+        <v>221</v>
       </c>
     </row>
     <row r="14">
@@ -1172,28 +1176,28 @@
         <v>0.05</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>-0.1</v>
+        <v>-0.04</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>-0.075</v>
+        <v>-0.045</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>-0.045</v>
+        <v>-0.027</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>-0.03</v>
+        <v>-0.018</v>
       </c>
       <c r="G14" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="H14" s="16" t="n">
-        <v>7552</v>
+        <v>8904</v>
       </c>
       <c r="I14" s="16" t="n">
-        <v>420</v>
+        <v>464</v>
       </c>
       <c r="J14" s="16" t="n">
-        <v>-629</v>
+        <v>-417</v>
       </c>
     </row>
     <row r="15">
@@ -1221,13 +1225,13 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="H15" s="16" t="n">
-        <v>6797</v>
+        <v>8013</v>
       </c>
       <c r="I15" s="16" t="n">
-        <v>529</v>
+        <v>623</v>
       </c>
       <c r="J15" s="16" t="n">
-        <v>-642</v>
+        <v>-757</v>
       </c>
     </row>
     <row r="16">
@@ -1240,28 +1244,28 @@
         <v>0.2</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>-0.08</v>
+        <v>-0.1</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>-0.08</v>
+        <v>-0.09</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>-0.048</v>
+        <v>-0.05400000000000001</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>-0.032</v>
+        <v>-0.036</v>
       </c>
       <c r="G16" s="21" t="n">
         <v>0.08</v>
       </c>
       <c r="H16" s="16" t="n">
-        <v>6253</v>
+        <v>7212</v>
       </c>
       <c r="I16" s="16" t="n">
-        <v>544</v>
+        <v>641</v>
       </c>
       <c r="J16" s="16" t="n">
-        <v>-544</v>
+        <v>-721</v>
       </c>
     </row>
     <row r="18">
@@ -1342,28 +1346,28 @@
         <v>0</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>-0.06</v>
+        <v>-0.05</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>-0.03</v>
+        <v>-0.025</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>-0.018</v>
+        <v>-0.015</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>-0.012</v>
+        <v>-0.01</v>
       </c>
       <c r="G20" s="21" t="n">
         <v>0</v>
       </c>
       <c r="H20" s="16" t="n">
-        <v>8303</v>
+        <v>8391</v>
       </c>
       <c r="I20" s="16" t="n">
         <v>0</v>
       </c>
       <c r="J20" s="16" t="n">
-        <v>-265</v>
+        <v>-221</v>
       </c>
     </row>
     <row r="21">
@@ -1391,13 +1395,13 @@
         <v>0.03</v>
       </c>
       <c r="H21" s="16" t="n">
-        <v>7473</v>
+        <v>7552</v>
       </c>
       <c r="I21" s="16" t="n">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="J21" s="16" t="n">
-        <v>-540</v>
+        <v>-545</v>
       </c>
     </row>
     <row r="22">
@@ -1410,28 +1414,28 @@
         <v>0.08</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>-0.1</v>
+        <v>-0.11</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>-0.075</v>
+        <v>-0.08</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>-0.045</v>
+        <v>-0.048</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>-0.03</v>
+        <v>-0.032</v>
       </c>
       <c r="G22" s="21" t="n">
         <v>0.05</v>
       </c>
       <c r="H22" s="16" t="n">
-        <v>6725</v>
+        <v>6721</v>
       </c>
       <c r="I22" s="16" t="n">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="J22" s="16" t="n">
-        <v>-560</v>
+        <v>-604</v>
       </c>
     </row>
     <row r="23">
@@ -1444,28 +1448,28 @@
         <v>0.15</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>-0.08</v>
+        <v>-0.1</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>-0.075</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>-0.045</v>
+        <v>-0.051</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>-0.03</v>
+        <v>-0.034</v>
       </c>
       <c r="G23" s="21" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="H23" s="16" t="n">
-        <v>6187</v>
+        <v>6049</v>
       </c>
       <c r="I23" s="16" t="n">
         <v>471</v>
       </c>
       <c r="J23" s="16" t="n">
-        <v>-504</v>
+        <v>-571</v>
       </c>
     </row>
   </sheetData>
@@ -1549,22 +1553,22 @@
         </is>
       </c>
       <c r="B5" s="25" t="n">
-        <v>248.18</v>
+        <v>253.52</v>
       </c>
       <c r="C5" s="25" t="n">
-        <v>278.37</v>
+        <v>284.38</v>
       </c>
       <c r="D5" s="25" t="n">
-        <v>308.56</v>
+        <v>315.25</v>
       </c>
       <c r="E5" s="26" t="n">
-        <v>338.76</v>
+        <v>346.11</v>
       </c>
       <c r="F5" s="26" t="n">
-        <v>368.95</v>
+        <v>376.97</v>
       </c>
       <c r="G5" s="26" t="n">
-        <v>399.15</v>
+        <v>407.83</v>
       </c>
     </row>
     <row r="6">
@@ -1574,22 +1578,22 @@
         </is>
       </c>
       <c r="B6" s="25" t="n">
-        <v>271.18</v>
+        <v>277.04</v>
       </c>
       <c r="C6" s="25" t="n">
-        <v>304.25</v>
+        <v>310.84</v>
       </c>
       <c r="D6" s="26" t="n">
-        <v>337.32</v>
+        <v>344.64</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>370.39</v>
+        <v>378.44</v>
       </c>
       <c r="F6" s="26" t="n">
-        <v>403.46</v>
+        <v>412.24</v>
       </c>
       <c r="G6" s="26" t="n">
-        <v>436.53</v>
+        <v>446.04</v>
       </c>
     </row>
     <row r="7">
@@ -1599,22 +1603,22 @@
         </is>
       </c>
       <c r="B7" s="25" t="n">
-        <v>294.19</v>
+        <v>300.55</v>
       </c>
       <c r="C7" s="26" t="n">
-        <v>330.13</v>
+        <v>337.29</v>
       </c>
       <c r="D7" s="26" t="n">
-        <v>366.08</v>
+        <v>374.03</v>
       </c>
       <c r="E7" s="26" t="n">
-        <v>402.02</v>
+        <v>410.77</v>
       </c>
       <c r="F7" s="26" t="n">
-        <v>437.97</v>
+        <v>447.51</v>
       </c>
       <c r="G7" s="26" t="n">
-        <v>473.91</v>
+        <v>484.26</v>
       </c>
     </row>
     <row r="8">
@@ -1623,23 +1627,23 @@
           <t>+10%</t>
         </is>
       </c>
-      <c r="B8" s="25" t="n">
-        <v>317.19</v>
+      <c r="B8" s="26" t="n">
+        <v>324.06</v>
       </c>
       <c r="C8" s="26" t="n">
-        <v>356.01</v>
+        <v>363.74</v>
       </c>
       <c r="D8" s="26" t="n">
-        <v>394.83</v>
+        <v>403.42</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>433.66</v>
+        <v>443.11</v>
       </c>
       <c r="F8" s="26" t="n">
-        <v>472.48</v>
+        <v>482.79</v>
       </c>
       <c r="G8" s="26" t="n">
-        <v>511.3</v>
+        <v>522.47</v>
       </c>
     </row>
     <row r="9">
@@ -1649,22 +1653,22 @@
         </is>
       </c>
       <c r="B9" s="26" t="n">
-        <v>340.2</v>
+        <v>347.58</v>
       </c>
       <c r="C9" s="26" t="n">
-        <v>381.89</v>
+        <v>390.2</v>
       </c>
       <c r="D9" s="26" t="n">
-        <v>423.59</v>
+        <v>432.82</v>
       </c>
       <c r="E9" s="26" t="n">
-        <v>465.29</v>
+        <v>475.44</v>
       </c>
       <c r="F9" s="26" t="n">
-        <v>506.99</v>
+        <v>518.0599999999999</v>
       </c>
       <c r="G9" s="26" t="n">
-        <v>548.6799999999999</v>
+        <v>560.6799999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2095,6 +2099,1467 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G54"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Three-stream revenue build (Core ARR / AI ARR / Services)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>FY26 base ($M):</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Core ARR $8,433  |  AI ARR $400  |  Services $719  |  Total $9,552</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Good AI</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="11" t="n"/>
+      <c r="G5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>$M unless noted</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FY29</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>FY30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Core ARR</t>
+        </is>
+      </c>
+      <c r="B7" s="16" t="n">
+        <v>9529</v>
+      </c>
+      <c r="C7" s="16" t="n">
+        <v>10863</v>
+      </c>
+      <c r="D7" s="16" t="n">
+        <v>12493</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>14117</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>AI ARR booked</t>
+        </is>
+      </c>
+      <c r="B8" s="16" t="n">
+        <v>800</v>
+      </c>
+      <c r="C8" s="16" t="n">
+        <v>1440</v>
+      </c>
+      <c r="D8" s="16" t="n">
+        <v>2304</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>3226</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>AI ARR recognized</t>
+        </is>
+      </c>
+      <c r="B9" s="17" t="n">
+        <v>560</v>
+      </c>
+      <c r="C9" s="17" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D9" s="17" t="n">
+        <v>2143</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>3152</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>AI deferred balance</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>240</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>480</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>641</v>
+      </c>
+      <c r="E10" s="13" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>712</v>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>698</v>
+      </c>
+      <c r="D11" s="16" t="n">
+        <v>698</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
+        <v>10801</v>
+      </c>
+      <c r="C12" s="17" t="n">
+        <v>12761</v>
+      </c>
+      <c r="D12" s="17" t="n">
+        <v>15334</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>17981</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Core ARR GM %</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="C13" s="7" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="D13" s="7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E13" s="7" t="n">
+        <v>0.845</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>AI ARR GM %</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C14" s="7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D14" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E14" s="7" t="n">
+        <v>0.65</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Services GM %</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C15" s="7" t="n">
+        <v>-0.08</v>
+      </c>
+      <c r="D15" s="7" t="n">
+        <v>-0.05</v>
+      </c>
+      <c r="E15" s="7" t="n">
+        <v>-0.02</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Blended GM %</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.749</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0.7582</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.766</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0.7766</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>GP Core ARR</t>
+        </is>
+      </c>
+      <c r="B17" s="13" t="n">
+        <v>7881</v>
+      </c>
+      <c r="C17" s="13" t="n">
+        <v>9071</v>
+      </c>
+      <c r="D17" s="13" t="n">
+        <v>10494</v>
+      </c>
+      <c r="E17" s="13" t="n">
+        <v>11929</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>GP AI ARR</t>
+        </is>
+      </c>
+      <c r="B18" s="13" t="n">
+        <v>280</v>
+      </c>
+      <c r="C18" s="13" t="n">
+        <v>660</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <v>1286</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <v>2049</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>GP Services</t>
+        </is>
+      </c>
+      <c r="B19" s="13" t="n">
+        <v>-71</v>
+      </c>
+      <c r="C19" s="13" t="n">
+        <v>-56</v>
+      </c>
+      <c r="D19" s="13" t="n">
+        <v>-35</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <v>-14</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Total GP</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="n">
+        <v>8090</v>
+      </c>
+      <c r="C20" s="15" t="n">
+        <v>9675</v>
+      </c>
+      <c r="D20" s="15" t="n">
+        <v>11745</v>
+      </c>
+      <c r="E20" s="15" t="n">
+        <v>13964</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Runs For Cash</t>
+        </is>
+      </c>
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>$M unless noted</t>
+        </is>
+      </c>
+      <c r="B23" s="4" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>FY29</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>FY30</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Core ARR</t>
+        </is>
+      </c>
+      <c r="B24" s="16" t="n">
+        <v>8855</v>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>8500</v>
+      </c>
+      <c r="D24" s="16" t="n">
+        <v>7650</v>
+      </c>
+      <c r="E24" s="16" t="n">
+        <v>6885</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>AI ARR booked</t>
+        </is>
+      </c>
+      <c r="B25" s="16" t="n">
+        <v>520</v>
+      </c>
+      <c r="C25" s="16" t="n">
+        <v>598</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>628</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>AI ARR recognized</t>
+        </is>
+      </c>
+      <c r="B26" s="17" t="n">
+        <v>416</v>
+      </c>
+      <c r="C26" s="17" t="n">
+        <v>560</v>
+      </c>
+      <c r="D26" s="17" t="n">
+        <v>662</v>
+      </c>
+      <c r="E26" s="17" t="n">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>AI deferred balance</t>
+        </is>
+      </c>
+      <c r="B27" s="13" t="n">
+        <v>104</v>
+      </c>
+      <c r="C27" s="13" t="n">
+        <v>142</v>
+      </c>
+      <c r="D27" s="13" t="n">
+        <v>108</v>
+      </c>
+      <c r="E27" s="13" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="B28" s="16" t="n">
+        <v>697</v>
+      </c>
+      <c r="C28" s="16" t="n">
+        <v>628</v>
+      </c>
+      <c r="D28" s="16" t="n">
+        <v>552</v>
+      </c>
+      <c r="E28" s="16" t="n">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B29" s="17" t="n">
+        <v>9968</v>
+      </c>
+      <c r="C29" s="17" t="n">
+        <v>9688</v>
+      </c>
+      <c r="D29" s="17" t="n">
+        <v>8865</v>
+      </c>
+      <c r="E29" s="17" t="n">
+        <v>8013</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Core ARR GM %</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="C30" s="7" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="D30" s="7" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E30" s="7" t="n">
+        <v>0.86</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>AI ARR GM %</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C31" s="7" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D31" s="7" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E31" s="7" t="n">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Services GM %</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C32" s="7" t="n">
+        <v>-0.12</v>
+      </c>
+      <c r="D32" s="7" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="E32" s="7" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Blended GM %</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="n">
+        <v>0.7464</v>
+      </c>
+      <c r="C33" s="7" t="n">
+        <v>0.7552</v>
+      </c>
+      <c r="D33" s="7" t="n">
+        <v>0.7591</v>
+      </c>
+      <c r="E33" s="7" t="n">
+        <v>0.7659</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>GP Core ARR</t>
+        </is>
+      </c>
+      <c r="B34" s="13" t="n">
+        <v>7323</v>
+      </c>
+      <c r="C34" s="13" t="n">
+        <v>7140</v>
+      </c>
+      <c r="D34" s="13" t="n">
+        <v>6503</v>
+      </c>
+      <c r="E34" s="13" t="n">
+        <v>5921</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>GP AI ARR</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="n">
+        <v>187</v>
+      </c>
+      <c r="C35" s="13" t="n">
+        <v>252</v>
+      </c>
+      <c r="D35" s="13" t="n">
+        <v>298</v>
+      </c>
+      <c r="E35" s="13" t="n">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t>GP Services</t>
+        </is>
+      </c>
+      <c r="B36" s="13" t="n">
+        <v>-70</v>
+      </c>
+      <c r="C36" s="13" t="n">
+        <v>-75</v>
+      </c>
+      <c r="D36" s="13" t="n">
+        <v>-72</v>
+      </c>
+      <c r="E36" s="13" t="n">
+        <v>-73</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>Total GP</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="n">
+        <v>7440</v>
+      </c>
+      <c r="C37" s="15" t="n">
+        <v>7317</v>
+      </c>
+      <c r="D37" s="15" t="n">
+        <v>6729</v>
+      </c>
+      <c r="E37" s="15" t="n">
+        <v>6137</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>What Goes Wrong</t>
+        </is>
+      </c>
+      <c r="B39" s="11" t="n"/>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="11" t="n"/>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>$M unless noted</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>FY29</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>FY30</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>Core ARR</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="n">
+        <v>8011</v>
+      </c>
+      <c r="C41" s="16" t="n">
+        <v>7210</v>
+      </c>
+      <c r="D41" s="16" t="n">
+        <v>6417</v>
+      </c>
+      <c r="E41" s="16" t="n">
+        <v>5775</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>AI ARR booked</t>
+        </is>
+      </c>
+      <c r="B42" s="16" t="n">
+        <v>480</v>
+      </c>
+      <c r="C42" s="16" t="n">
+        <v>528</v>
+      </c>
+      <c r="D42" s="16" t="n">
+        <v>554</v>
+      </c>
+      <c r="E42" s="16" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>AI ARR recognized</t>
+        </is>
+      </c>
+      <c r="B43" s="17" t="n">
+        <v>408</v>
+      </c>
+      <c r="C43" s="17" t="n">
+        <v>511</v>
+      </c>
+      <c r="D43" s="17" t="n">
+        <v>589</v>
+      </c>
+      <c r="E43" s="17" t="n">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>AI deferred balance</t>
+        </is>
+      </c>
+      <c r="B44" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="C44" s="13" t="n">
+        <v>89</v>
+      </c>
+      <c r="D44" s="13" t="n">
+        <v>54</v>
+      </c>
+      <c r="E44" s="13" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>Services</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="n">
+        <v>647</v>
+      </c>
+      <c r="C45" s="16" t="n">
+        <v>550</v>
+      </c>
+      <c r="D45" s="16" t="n">
+        <v>468</v>
+      </c>
+      <c r="E45" s="16" t="n">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Total revenue</t>
+        </is>
+      </c>
+      <c r="B46" s="17" t="n">
+        <v>9066</v>
+      </c>
+      <c r="C46" s="17" t="n">
+        <v>8271</v>
+      </c>
+      <c r="D46" s="17" t="n">
+        <v>7474</v>
+      </c>
+      <c r="E46" s="17" t="n">
+        <v>6754</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Core ARR GM %</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="n">
+        <v>0.827</v>
+      </c>
+      <c r="C47" s="7" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="D47" s="7" t="n">
+        <v>0.835</v>
+      </c>
+      <c r="E47" s="7" t="n">
+        <v>0.84</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>AI ARR GM %</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="C48" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D48" s="7" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="E48" s="7" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Services GM %</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="C49" s="7" t="n">
+        <v>-0.13</v>
+      </c>
+      <c r="D49" s="7" t="n">
+        <v>-0.16</v>
+      </c>
+      <c r="E49" s="7" t="n">
+        <v>-0.18</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Blended GM %</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="n">
+        <v>0.7416</v>
+      </c>
+      <c r="C50" s="7" t="n">
+        <v>0.7396</v>
+      </c>
+      <c r="D50" s="7" t="n">
+        <v>0.7385</v>
+      </c>
+      <c r="E50" s="7" t="n">
+        <v>0.7409</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="12" t="inlineStr">
+        <is>
+          <t>GP Core ARR</t>
+        </is>
+      </c>
+      <c r="B51" s="13" t="n">
+        <v>6625</v>
+      </c>
+      <c r="C51" s="13" t="n">
+        <v>5984</v>
+      </c>
+      <c r="D51" s="13" t="n">
+        <v>5358</v>
+      </c>
+      <c r="E51" s="13" t="n">
+        <v>4851</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="12" t="inlineStr">
+        <is>
+          <t>GP AI ARR</t>
+        </is>
+      </c>
+      <c r="B52" s="13" t="n">
+        <v>163</v>
+      </c>
+      <c r="C52" s="13" t="n">
+        <v>204</v>
+      </c>
+      <c r="D52" s="13" t="n">
+        <v>236</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="12" t="inlineStr">
+        <is>
+          <t>GP Services</t>
+        </is>
+      </c>
+      <c r="B53" s="13" t="n">
+        <v>-65</v>
+      </c>
+      <c r="C53" s="13" t="n">
+        <v>-72</v>
+      </c>
+      <c r="D53" s="13" t="n">
+        <v>-75</v>
+      </c>
+      <c r="E53" s="13" t="n">
+        <v>-74</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Total GP</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="n">
+        <v>6724</v>
+      </c>
+      <c r="C54" s="15" t="n">
+        <v>6117</v>
+      </c>
+      <c r="D54" s="15" t="n">
+        <v>5519</v>
+      </c>
+      <c r="E54" s="15" t="n">
+        <v>5004</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>AI ARR — booked vs recognized (deferred-revenue mechanic)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AI ARR has a per-year deferred fraction. Deferred dollars sit on the balance sheet and are recognized ratably over the next two years (50%/50%). Total revenue uses RECOGNIZED, not booked.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>FY26 base AI ARR: $400M  (per Q4 FY26 prepared remarks)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Good AI</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n"/>
+      <c r="C5" s="11" t="n"/>
+      <c r="D5" s="11" t="n"/>
+      <c r="E5" s="11" t="n"/>
+      <c r="F5" s="11" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>$M / %</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>FY29</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>FY30</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>Booked growth %</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="E7" s="7" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>Deferred fraction %</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D8" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>AI ARR booked ($M)</t>
+        </is>
+      </c>
+      <c r="B9" s="16" t="n">
+        <v>800</v>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>1440</v>
+      </c>
+      <c r="D9" s="16" t="n">
+        <v>2304</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>3226</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>AI ARR recognized ($M)</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="n">
+        <v>560</v>
+      </c>
+      <c r="C10" s="17" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D10" s="17" t="n">
+        <v>2143</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>3152</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Deferred balance ($M)</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="n">
+        <v>240</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>480</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>641</v>
+      </c>
+      <c r="E11" s="13" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>Booked − Recognized</t>
+        </is>
+      </c>
+      <c r="B12" s="27" t="n">
+        <v>240</v>
+      </c>
+      <c r="C12" s="27" t="n">
+        <v>240</v>
+      </c>
+      <c r="D12" s="27" t="n">
+        <v>161</v>
+      </c>
+      <c r="E12" s="27" t="n">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Runs For Cash</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>$M / %</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>FY29</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>FY30</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Booked growth %</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C16" s="7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D16" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E16" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Deferred fraction %</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C17" s="7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D17" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E17" s="7" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>AI ARR booked ($M)</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="n">
+        <v>520</v>
+      </c>
+      <c r="C18" s="16" t="n">
+        <v>598</v>
+      </c>
+      <c r="D18" s="16" t="n">
+        <v>628</v>
+      </c>
+      <c r="E18" s="16" t="n">
+        <v>628</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>AI ARR recognized ($M)</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>416</v>
+      </c>
+      <c r="C19" s="17" t="n">
+        <v>560</v>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>662</v>
+      </c>
+      <c r="E19" s="17" t="n">
+        <v>641</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Deferred balance ($M)</t>
+        </is>
+      </c>
+      <c r="B20" s="13" t="n">
+        <v>104</v>
+      </c>
+      <c r="C20" s="13" t="n">
+        <v>142</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <v>108</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Booked − Recognized</t>
+        </is>
+      </c>
+      <c r="B21" s="27" t="n">
+        <v>104</v>
+      </c>
+      <c r="C21" s="27" t="n">
+        <v>38</v>
+      </c>
+      <c r="D21" s="27" t="n">
+        <v>-34</v>
+      </c>
+      <c r="E21" s="27" t="n">
+        <v>-13</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>What Goes Wrong</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="n"/>
+      <c r="C23" s="11" t="n"/>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
+      <c r="F23" s="11" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>$M / %</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>FY27</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>FY29</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>FY30</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Booked growth %</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C25" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D25" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E25" s="7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>Deferred fraction %</t>
+        </is>
+      </c>
+      <c r="B26" s="7" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C26" s="7" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D26" s="7" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="E26" s="7" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>AI ARR booked ($M)</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="n">
+        <v>480</v>
+      </c>
+      <c r="C27" s="16" t="n">
+        <v>528</v>
+      </c>
+      <c r="D27" s="16" t="n">
+        <v>554</v>
+      </c>
+      <c r="E27" s="16" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>AI ARR recognized ($M)</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="n">
+        <v>408</v>
+      </c>
+      <c r="C28" s="17" t="n">
+        <v>511</v>
+      </c>
+      <c r="D28" s="17" t="n">
+        <v>589</v>
+      </c>
+      <c r="E28" s="17" t="n">
+        <v>567</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>Deferred balance ($M)</t>
+        </is>
+      </c>
+      <c r="B29" s="13" t="n">
+        <v>72</v>
+      </c>
+      <c r="C29" s="13" t="n">
+        <v>89</v>
+      </c>
+      <c r="D29" s="13" t="n">
+        <v>54</v>
+      </c>
+      <c r="E29" s="13" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>Booked − Recognized</t>
+        </is>
+      </c>
+      <c r="B30" s="27" t="n">
+        <v>72</v>
+      </c>
+      <c r="C30" s="27" t="n">
+        <v>17</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>-35</v>
+      </c>
+      <c r="E30" s="27" t="n">
+        <v>-13</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -2218,16 +3683,16 @@
         </is>
       </c>
       <c r="C11" s="7" t="n">
-        <v>0.15</v>
+        <v>0.1308</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>0.17</v>
+        <v>0.1815</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>0.18</v>
+        <v>0.2016</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>0.16</v>
+        <v>0.1726</v>
       </c>
     </row>
     <row r="12">
@@ -2242,16 +3707,16 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>0.1</v>
+        <v>0.0436</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.0281</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>0.05</v>
+        <v>-0.08500000000000001</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>0.04</v>
+        <v>-0.0961</v>
       </c>
     </row>
     <row r="13">
@@ -2266,16 +3731,16 @@
         </is>
       </c>
       <c r="C13" s="7" t="n">
-        <v>0.08</v>
+        <v>-0.0509</v>
       </c>
       <c r="D13" s="7" t="n">
-        <v>0.04</v>
+        <v>-0.0877</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>0.01</v>
+        <v>-0.0964</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>-0.02</v>
+        <v>-0.0963</v>
       </c>
     </row>
     <row r="15">
@@ -2293,7 +3758,7 @@
         <v>0.16</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>0.18</v>
+        <v>0.1801</v>
       </c>
       <c r="E15" s="7" t="n">
         <v>0.19</v>
@@ -2314,16 +3779,16 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>0.1</v>
+        <v>-0.04</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.09</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>0.05</v>
+        <v>-0.1</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>0.04</v>
+        <v>-0.0801</v>
       </c>
     </row>
     <row r="17">
@@ -2338,16 +3803,16 @@
         </is>
       </c>
       <c r="C17" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>-0.05</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>0.03</v>
+        <v>-0.1</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>0</v>
+        <v>-0.11</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>-0.02</v>
+        <v>-0.08989999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -2362,16 +3827,16 @@
         </is>
       </c>
       <c r="C19" s="7" t="n">
-        <v>0.19</v>
+        <v>0.251</v>
       </c>
       <c r="D19" s="7" t="n">
-        <v>0.18</v>
+        <v>0.2418</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>0.17</v>
+        <v>0.234</v>
       </c>
       <c r="F19" s="7" t="n">
-        <v>0.16</v>
+        <v>0.2234</v>
       </c>
     </row>
     <row r="20">
@@ -2386,16 +3851,16 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>0.19</v>
+        <v>0.2536</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>0.18</v>
+        <v>0.2448</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>0.17</v>
+        <v>0.2409</v>
       </c>
       <c r="F20" s="7" t="n">
-        <v>0.16</v>
+        <v>0.2341</v>
       </c>
     </row>
     <row r="21">
@@ -2410,16 +3875,16 @@
         </is>
       </c>
       <c r="C21" s="7" t="n">
-        <v>0.2</v>
+        <v>0.2584</v>
       </c>
       <c r="D21" s="7" t="n">
-        <v>0.2</v>
+        <v>0.2604</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>0.21</v>
+        <v>0.2615</v>
       </c>
       <c r="F21" s="7" t="n">
-        <v>0.22</v>
+        <v>0.2591</v>
       </c>
     </row>
     <row r="23">
@@ -2434,16 +3899,16 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>0.27</v>
+        <v>0.26</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
     </row>
     <row r="24">
@@ -2458,16 +3923,16 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>0.24</v>
+        <v>0.2</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="25">
@@ -2482,16 +3947,16 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>0.28</v>
+        <v>0.26</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>0.28</v>
+        <v>0.23</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>0.27</v>
+        <v>0.2</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>0.27</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="27">
@@ -2506,16 +3971,16 @@
         </is>
       </c>
       <c r="C27" s="7" t="n">
-        <v>0.26</v>
+        <v>0.25</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="28">
@@ -2530,16 +3995,16 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>0.26</v>
+        <v>0.22</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>0.2</v>
+        <v>0.1299</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="29">
@@ -2554,16 +4019,16 @@
         </is>
       </c>
       <c r="C29" s="7" t="n">
-        <v>0.28</v>
+        <v>0.24</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>0.28</v>
+        <v>0.21</v>
       </c>
       <c r="E29" s="7" t="n">
-        <v>0.27</v>
+        <v>0.18</v>
       </c>
       <c r="F29" s="7" t="n">
-        <v>0.26</v>
+        <v>0.1601</v>
       </c>
     </row>
     <row r="31">
@@ -2602,16 +4067,16 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>0.08</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>0.075</v>
+        <v>0.06</v>
       </c>
       <c r="F32" s="7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="33">
@@ -2629,13 +4094,13 @@
         <v>0.09</v>
       </c>
       <c r="D33" s="7" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>0.09</v>
+        <v>0.0751</v>
       </c>
       <c r="F33" s="7" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -2650,16 +4115,16 @@
         </is>
       </c>
       <c r="C35" s="7" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="D35" s="7" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>0.14</v>
+        <v>0.12</v>
       </c>
       <c r="F35" s="7" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="36">
@@ -2674,16 +4139,16 @@
         </is>
       </c>
       <c r="C36" s="7" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="D36" s="7" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="F36" s="7" t="n">
-        <v>0.1</v>
+        <v>0.0401</v>
       </c>
     </row>
     <row r="37">
@@ -2698,16 +4163,16 @@
         </is>
       </c>
       <c r="C37" s="7" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="D37" s="7" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="F37" s="7" t="n">
-        <v>0.13</v>
+        <v>0.0999</v>
       </c>
     </row>
     <row r="39">
@@ -2722,16 +4187,16 @@
         </is>
       </c>
       <c r="C39" s="7" t="n">
-        <v>0.32</v>
+        <v>0.33</v>
       </c>
       <c r="D39" s="7" t="n">
-        <v>0.34</v>
+        <v>0.35</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>0.36</v>
+        <v>0.37</v>
       </c>
       <c r="F39" s="7" t="n">
-        <v>0.37</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="40">
@@ -2752,10 +4217,10 @@
         <v>0.36</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>0.38</v>
+        <v>0.36</v>
       </c>
       <c r="F40" s="7" t="n">
-        <v>0.4</v>
+        <v>0.3399</v>
       </c>
     </row>
     <row r="41">
@@ -2776,10 +4241,10 @@
         <v>0.3</v>
       </c>
       <c r="E41" s="7" t="n">
-        <v>0.3</v>
+        <v>0.28</v>
       </c>
       <c r="F41" s="7" t="n">
-        <v>0.3</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="43">
@@ -2794,16 +4259,16 @@
         </is>
       </c>
       <c r="C43" s="7" t="n">
-        <v>0.015</v>
+        <v>0.0201</v>
       </c>
       <c r="D43" s="7" t="n">
-        <v>0.015</v>
+        <v>0.0198</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>0.02</v>
+        <v>0.0249</v>
       </c>
       <c r="F43" s="7" t="n">
-        <v>0.02</v>
+        <v>0.0251</v>
       </c>
     </row>
     <row r="44">
@@ -2818,16 +4283,16 @@
         </is>
       </c>
       <c r="C44" s="7" t="n">
-        <v>0.035</v>
+        <v>0.0399</v>
       </c>
       <c r="D44" s="7" t="n">
-        <v>0.05</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>0.055</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="F44" s="7" t="n">
-        <v>0.05</v>
+        <v>0.0997</v>
       </c>
     </row>
     <row r="45">
@@ -2842,16 +4307,16 @@
         </is>
       </c>
       <c r="C45" s="7" t="n">
-        <v>0.02</v>
+        <v>0.025</v>
       </c>
       <c r="D45" s="7" t="n">
-        <v>0.02</v>
+        <v>0.0348</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>0.025</v>
+        <v>0.04</v>
       </c>
       <c r="F45" s="7" t="n">
-        <v>0.025</v>
+        <v>0.0401</v>
       </c>
     </row>
     <row r="47">
@@ -2866,7 +4331,7 @@
         </is>
       </c>
       <c r="C47" s="9" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48">
@@ -2876,7 +4341,7 @@
         </is>
       </c>
       <c r="C48" s="9" t="n">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="49">
@@ -2886,7 +4351,7 @@
         </is>
       </c>
       <c r="C49" s="9" t="n">
-        <v>3</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="50">
@@ -2901,7 +4366,7 @@
         </is>
       </c>
       <c r="C50" s="10" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
     </row>
     <row r="51">
@@ -2911,7 +4376,7 @@
         </is>
       </c>
       <c r="C51" s="10" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="52">
@@ -2921,7 +4386,7 @@
         </is>
       </c>
       <c r="C52" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="53">
@@ -2936,7 +4401,7 @@
         </is>
       </c>
       <c r="C53" s="5" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="54">
@@ -2946,7 +4411,7 @@
         </is>
       </c>
       <c r="C54" s="5" t="n">
-        <v>0.45</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="55">
@@ -2956,7 +4421,7 @@
         </is>
       </c>
       <c r="C55" s="5" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>
@@ -5956,7 +7421,7 @@
         <v/>
       </c>
       <c r="C4" s="19" t="n">
-        <v>572.04</v>
+        <v>728.29</v>
       </c>
       <c r="D4" s="7">
         <f>C4/129.34-1</f>
@@ -5982,7 +7447,7 @@
         <v/>
       </c>
       <c r="C5" s="19" t="n">
-        <v>106.62</v>
+        <v>124.18</v>
       </c>
       <c r="D5" s="7">
         <f>C5/129.34-1</f>
@@ -6008,7 +7473,7 @@
         <v/>
       </c>
       <c r="C6" s="19" t="n">
-        <v>68.01000000000001</v>
+        <v>68.23</v>
       </c>
       <c r="D6" s="7">
         <f>C6/129.34-1</f>
@@ -6379,10 +7844,10 @@
         </is>
       </c>
       <c r="D5" s="6" t="n">
-        <v>468.37</v>
+        <v>592.42</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>2.621</v>
+        <v>3.58</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -6393,10 +7858,10 @@
         <v>0.068</v>
       </c>
       <c r="H5" s="21" t="n">
-        <v>2.621</v>
+        <v>3.58</v>
       </c>
       <c r="I5" s="7" t="n">
-        <v>0.536</v>
+        <v>0.6609999999999999</v>
       </c>
       <c r="J5" s="18" t="n">
         <v>268</v>
@@ -6420,10 +7885,10 @@
         </is>
       </c>
       <c r="D6" s="6" t="n">
-        <v>572.04</v>
+        <v>728.29</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>3.423</v>
+        <v>4.631</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -6434,10 +7899,10 @@
         <v>0.095</v>
       </c>
       <c r="H6" s="21" t="n">
-        <v>3.423</v>
+        <v>4.631</v>
       </c>
       <c r="I6" s="7" t="n">
-        <v>0.45</v>
+        <v>0.54</v>
       </c>
       <c r="J6" s="18" t="n">
         <v>268</v>
@@ -6461,30 +7926,30 @@
         </is>
       </c>
       <c r="D7" s="6" t="n">
-        <v>111.25</v>
+        <v>125.57</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>-0.14</v>
+        <v>-0.029</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>7.8% ($10.04)</t>
+          <t>9.2% ($11.93)</t>
         </is>
       </c>
       <c r="G7" s="7" t="n">
-        <v>0.192</v>
+        <v>0.231</v>
       </c>
       <c r="H7" s="21" t="n">
-        <v>-0.062</v>
+        <v>0.063</v>
       </c>
       <c r="I7" s="7" t="n">
-        <v>-0.021</v>
+        <v>0.021</v>
       </c>
       <c r="J7" s="18" t="n">
         <v>268</v>
       </c>
       <c r="K7" s="18" t="n">
-        <v>224.9</v>
+        <v>217.7</v>
       </c>
     </row>
     <row r="8">
@@ -6502,30 +7967,30 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>106.62</v>
+        <v>124.18</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>-0.176</v>
+        <v>-0.04</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>12.2% ($15.81)</t>
+          <t>14.7% ($19.00)</t>
         </is>
       </c>
       <c r="G8" s="7" t="n">
-        <v>0.268</v>
+        <v>0.367</v>
       </c>
       <c r="H8" s="21" t="n">
-        <v>-0.053</v>
+        <v>0.107</v>
       </c>
       <c r="I8" s="7" t="n">
-        <v>-0.014</v>
+        <v>0.026</v>
       </c>
       <c r="J8" s="18" t="n">
         <v>268</v>
       </c>
       <c r="K8" s="18" t="n">
-        <v>211.4</v>
+        <v>196</v>
       </c>
     </row>
     <row r="9">
@@ -6543,24 +8008,24 @@
         </is>
       </c>
       <c r="D9" s="6" t="n">
-        <v>72.90000000000001</v>
+        <v>73.65000000000001</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>-0.436</v>
+        <v>-0.431</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2.5% ($3.17)</t>
+          <t>2.5% ($3.26)</t>
         </is>
       </c>
       <c r="G9" s="7" t="n">
         <v>0.107</v>
       </c>
       <c r="H9" s="21" t="n">
-        <v>-0.412</v>
+        <v>-0.405</v>
       </c>
       <c r="I9" s="7" t="n">
-        <v>-0.162</v>
+        <v>-0.159</v>
       </c>
       <c r="J9" s="18" t="n">
         <v>268</v>
@@ -6584,24 +8049,24 @@
         </is>
       </c>
       <c r="D10" s="6" t="n">
-        <v>68.01000000000001</v>
+        <v>68.23</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>-0.474</v>
+        <v>-0.472</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>4.0% ($5.16)</t>
+          <t>4.1% ($5.27)</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
         <v>0.153</v>
       </c>
       <c r="H10" s="21" t="n">
-        <v>-0.434</v>
+        <v>-0.4320000000000001</v>
       </c>
       <c r="I10" s="7" t="n">
-        <v>-0.133</v>
+        <v>-0.132</v>
       </c>
       <c r="J10" s="18" t="n">
         <v>268</v>
@@ -6617,7 +8082,7 @@
         </is>
       </c>
       <c r="H12" s="21" t="n">
-        <v>0.772</v>
+        <v>1.154</v>
       </c>
     </row>
     <row r="13">
@@ -6627,7 +8092,7 @@
         </is>
       </c>
       <c r="H13" s="21" t="n">
-        <v>1.049</v>
+        <v>1.529</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix AI ARR base double-count: subtract from HCM/Fin so 4 streams sum to reported FY26 $9.55B
</commit_message>
<xml_diff>
--- a/WDAY_Model.xlsx
+++ b/WDAY_Model.xlsx
@@ -747,7 +747,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>+120.7%</t>
+          <t>+115.3%</t>
         </is>
       </c>
     </row>
@@ -759,7 +759,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>+158.2%</t>
+          <t>+151.8%</t>
         </is>
       </c>
     </row>
@@ -822,10 +822,10 @@
         <v>0.35</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>605.53</v>
+        <v>590.6900000000001</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>476.19</v>
+        <v>461.35</v>
       </c>
       <c r="E22" s="6" t="n">
         <v>0</v>
@@ -834,10 +834,10 @@
         <v>5652</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>3.682</v>
+        <v>3.567</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>0.6729999999999999</v>
+        <v>0.659</v>
       </c>
     </row>
     <row r="23">
@@ -850,22 +850,22 @@
         <v>0.35</v>
       </c>
       <c r="C23" s="6" t="n">
-        <v>129.83</v>
+        <v>126.56</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>0.49</v>
+        <v>-2.78</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>12.71</v>
+        <v>12.08</v>
       </c>
       <c r="F23" s="8" t="n">
         <v>6617</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>0.102</v>
+        <v>0.07200000000000001</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>0.033</v>
+        <v>0.023</v>
       </c>
     </row>
     <row r="24">
@@ -878,22 +878,22 @@
         <v>0.3</v>
       </c>
       <c r="C24" s="6" t="n">
-        <v>75.38</v>
+        <v>73.92</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>-53.96</v>
+        <v>-55.42</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>3.46</v>
+        <v>3.29</v>
       </c>
       <c r="F24" s="8" t="n">
         <v>2970</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>-0.39</v>
+        <v>-0.403</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>-0.152</v>
+        <v>-0.158</v>
       </c>
     </row>
     <row r="26">
@@ -955,10 +955,10 @@
         <v>0.35</v>
       </c>
       <c r="C28" s="6" t="n">
-        <v>740.9299999999999</v>
+        <v>722.85</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>611.59</v>
+        <v>593.51</v>
       </c>
       <c r="E28" s="6" t="n">
         <v>0</v>
@@ -967,10 +967,10 @@
         <v>10044</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>4.729</v>
+        <v>4.589</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>0.547</v>
+        <v>0.5379999999999999</v>
       </c>
     </row>
     <row r="29">
@@ -983,22 +983,22 @@
         <v>0.35</v>
       </c>
       <c r="C29" s="6" t="n">
-        <v>128.2</v>
+        <v>125.12</v>
       </c>
       <c r="D29" s="7" t="n">
-        <v>-1.14</v>
+        <v>-4.22</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>20.26</v>
+        <v>19.26</v>
       </c>
       <c r="F29" s="8" t="n">
         <v>9556</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>0.148</v>
+        <v>0.116</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>0.035</v>
+        <v>0.028</v>
       </c>
     </row>
     <row r="30">
@@ -1011,22 +1011,22 @@
         <v>0.3</v>
       </c>
       <c r="C30" s="6" t="n">
-        <v>69.81</v>
+        <v>68.55</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>-59.53</v>
+        <v>-60.79</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>5.6</v>
+        <v>5.33</v>
       </c>
       <c r="F30" s="8" t="n">
         <v>3841</v>
       </c>
       <c r="G30" s="9" t="n">
-        <v>-0.417</v>
+        <v>-0.429</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>-0.126</v>
+        <v>-0.131</v>
       </c>
     </row>
     <row r="32">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>28x FCF on $22.32 FY29 FCF/share growing 18% = $606 + $22 cum cap return = TSR +368%</t>
+          <t>28x FCF on $21.26 FY29 FCF/share growing 18% = $591 + $22 cum cap return = TSR +357%</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>9x FCF on $14.79 FY29 FCF/share growing -8% = $130 + $39 cum cap return = TSR +10%</t>
+          <t>9x FCF on $14.06 FY29 FCF/share growing -8% = $127 + $38 cum cap return = TSR +7%</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>7x FCF on $8.52 FY29 FCF/share growing -9% = $75 + $15 cum cap return = TSR -39%</t>
+          <t>7x FCF on $8.11 FY29 FCF/share growing -9% = $74 + $15 cum cap return = TSR -40%</t>
         </is>
       </c>
     </row>
@@ -1195,28 +1195,28 @@
         <v>0</v>
       </c>
       <c r="C6" s="10" t="n">
-        <v>0.147</v>
+        <v>0.1466</v>
       </c>
       <c r="D6" s="10" t="n">
-        <v>0.0735</v>
+        <v>0.0733</v>
       </c>
       <c r="E6" s="10" t="n">
-        <v>0.0441</v>
+        <v>0.044</v>
       </c>
       <c r="F6" s="10" t="n">
-        <v>0.0294</v>
+        <v>0.0293</v>
       </c>
       <c r="G6" s="9" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="19" t="n">
-        <v>10132</v>
+        <v>10128</v>
       </c>
       <c r="I6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J6" s="19" t="n">
-        <v>649</v>
+        <v>647</v>
       </c>
     </row>
     <row r="7">
@@ -1229,13 +1229,13 @@
         <v>0.08</v>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.1337</v>
+        <v>0.1333</v>
       </c>
       <c r="D7" s="10" t="n">
-        <v>0.0268</v>
+        <v>0.0266</v>
       </c>
       <c r="E7" s="10" t="n">
-        <v>0.0161</v>
+        <v>0.016</v>
       </c>
       <c r="F7" s="10" t="n">
         <v>0.0107</v>
@@ -1244,13 +1244,13 @@
         <v>0.08</v>
       </c>
       <c r="H7" s="19" t="n">
-        <v>11486</v>
+        <v>11477</v>
       </c>
       <c r="I7" s="19" t="n">
-        <v>811</v>
+        <v>810</v>
       </c>
       <c r="J7" s="19" t="n">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="8">
@@ -1263,28 +1263,28 @@
         <v>0.18</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>0.1269</v>
+        <v>0.1266</v>
       </c>
       <c r="D8" s="10" t="n">
-        <v>0.0135</v>
+        <v>0.0133</v>
       </c>
       <c r="E8" s="10" t="n">
-        <v>0.008100000000000001</v>
+        <v>0.008</v>
       </c>
       <c r="F8" s="10" t="n">
-        <v>0.0054</v>
+        <v>0.0053</v>
       </c>
       <c r="G8" s="9" t="n">
         <v>0.1</v>
       </c>
       <c r="H8" s="19" t="n">
-        <v>12944</v>
+        <v>12930</v>
       </c>
       <c r="I8" s="19" t="n">
-        <v>1149</v>
+        <v>1148</v>
       </c>
       <c r="J8" s="19" t="n">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="9">
@@ -1297,13 +1297,13 @@
         <v>0.3</v>
       </c>
       <c r="C9" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.1133</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>-0.0032</v>
+        <v>-0.0034</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>-0.0019</v>
+        <v>-0.002</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>-0.0013</v>
@@ -1312,13 +1312,13 @@
         <v>0.12</v>
       </c>
       <c r="H9" s="19" t="n">
-        <v>14415</v>
+        <v>14395</v>
       </c>
       <c r="I9" s="19" t="n">
-        <v>1553</v>
+        <v>1552</v>
       </c>
       <c r="J9" s="19" t="n">
-        <v>-42</v>
+        <v>-43</v>
       </c>
     </row>
     <row r="11">
@@ -1402,7 +1402,7 @@
         <v>0.0533</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>0.0266</v>
+        <v>0.0267</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>0.016</v>
@@ -1414,13 +1414,13 @@
         <v>0</v>
       </c>
       <c r="H13" s="19" t="n">
-        <v>9303</v>
+        <v>9304</v>
       </c>
       <c r="I13" s="19" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="19" t="n">
-        <v>235</v>
+        <v>236</v>
       </c>
     </row>
     <row r="14">
@@ -1433,7 +1433,7 @@
         <v>0.05</v>
       </c>
       <c r="C14" s="10" t="n">
-        <v>-0.0335</v>
+        <v>-0.0333</v>
       </c>
       <c r="D14" s="10" t="n">
         <v>-0.0417</v>
@@ -1448,7 +1448,7 @@
         <v>0.05</v>
       </c>
       <c r="H14" s="19" t="n">
-        <v>8992</v>
+        <v>8994</v>
       </c>
       <c r="I14" s="19" t="n">
         <v>465</v>
@@ -1467,7 +1467,7 @@
         <v>0.12</v>
       </c>
       <c r="C15" s="10" t="n">
-        <v>-0.0935</v>
+        <v>-0.09329999999999999</v>
       </c>
       <c r="D15" s="10" t="n">
         <v>-0.08169999999999999</v>
@@ -1482,13 +1482,13 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="H15" s="19" t="n">
-        <v>8152</v>
+        <v>8155</v>
       </c>
       <c r="I15" s="19" t="n">
-        <v>629</v>
+        <v>630</v>
       </c>
       <c r="J15" s="19" t="n">
-        <v>-735</v>
+        <v>-734</v>
       </c>
     </row>
     <row r="16">
@@ -1516,7 +1516,7 @@
         <v>0.08</v>
       </c>
       <c r="H16" s="19" t="n">
-        <v>7336</v>
+        <v>7340</v>
       </c>
       <c r="I16" s="19" t="n">
         <v>652</v>
@@ -1606,7 +1606,7 @@
         <v>-0.0467</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>-0.0234</v>
+        <v>-0.0233</v>
       </c>
       <c r="E20" s="10" t="n">
         <v>-0.014</v>
@@ -1618,7 +1618,7 @@
         <v>0</v>
       </c>
       <c r="H20" s="19" t="n">
-        <v>8420</v>
+        <v>8421</v>
       </c>
       <c r="I20" s="19" t="n">
         <v>0</v>
@@ -1640,7 +1640,7 @@
         <v>-0.09669999999999999</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>-0.0634</v>
+        <v>-0.0633</v>
       </c>
       <c r="E21" s="10" t="n">
         <v>-0.038</v>
@@ -1652,13 +1652,13 @@
         <v>0.03</v>
       </c>
       <c r="H21" s="19" t="n">
-        <v>7606</v>
+        <v>7607</v>
       </c>
       <c r="I21" s="19" t="n">
         <v>253</v>
       </c>
       <c r="J21" s="19" t="n">
-        <v>-534</v>
+        <v>-533</v>
       </c>
     </row>
     <row r="22">
@@ -1674,7 +1674,7 @@
         <v>-0.1067</v>
       </c>
       <c r="D22" s="10" t="n">
-        <v>-0.0784</v>
+        <v>-0.07829999999999999</v>
       </c>
       <c r="E22" s="10" t="n">
         <v>-0.047</v>
@@ -1686,7 +1686,7 @@
         <v>0.05</v>
       </c>
       <c r="H22" s="19" t="n">
-        <v>6794</v>
+        <v>6796</v>
       </c>
       <c r="I22" s="19" t="n">
         <v>380</v>
@@ -1708,7 +1708,7 @@
         <v>-0.09669999999999999</v>
       </c>
       <c r="D23" s="10" t="n">
-        <v>-0.0834</v>
+        <v>-0.0833</v>
       </c>
       <c r="E23" s="10" t="n">
         <v>-0.05</v>
@@ -1720,7 +1720,7 @@
         <v>0.07000000000000001</v>
       </c>
       <c r="H23" s="19" t="n">
-        <v>6137</v>
+        <v>6139</v>
       </c>
       <c r="I23" s="19" t="n">
         <v>476</v>
@@ -1810,22 +1810,22 @@
         </is>
       </c>
       <c r="B5" s="38" t="n">
-        <v>261.74</v>
+        <v>250.01</v>
       </c>
       <c r="C5" s="38" t="n">
-        <v>293.63</v>
-      </c>
-      <c r="D5" s="39" t="n">
-        <v>325.52</v>
+        <v>280.43</v>
+      </c>
+      <c r="D5" s="38" t="n">
+        <v>310.86</v>
       </c>
       <c r="E5" s="39" t="n">
-        <v>357.4</v>
+        <v>341.28</v>
       </c>
       <c r="F5" s="39" t="n">
-        <v>389.29</v>
+        <v>371.7</v>
       </c>
       <c r="G5" s="39" t="n">
-        <v>421.18</v>
+        <v>402.13</v>
       </c>
     </row>
     <row r="6">
@@ -1835,22 +1835,22 @@
         </is>
       </c>
       <c r="B6" s="38" t="n">
-        <v>286.03</v>
+        <v>273.19</v>
       </c>
       <c r="C6" s="38" t="n">
-        <v>320.96</v>
+        <v>306.51</v>
       </c>
       <c r="D6" s="39" t="n">
-        <v>355.88</v>
+        <v>339.83</v>
       </c>
       <c r="E6" s="39" t="n">
-        <v>390.81</v>
+        <v>373.15</v>
       </c>
       <c r="F6" s="39" t="n">
-        <v>425.73</v>
+        <v>406.47</v>
       </c>
       <c r="G6" s="39" t="n">
-        <v>460.66</v>
+        <v>439.79</v>
       </c>
     </row>
     <row r="7">
@@ -1860,22 +1860,22 @@
         </is>
       </c>
       <c r="B7" s="38" t="n">
-        <v>310.32</v>
+        <v>296.36</v>
       </c>
       <c r="C7" s="39" t="n">
-        <v>348.29</v>
+        <v>332.58</v>
       </c>
       <c r="D7" s="39" t="n">
-        <v>386.25</v>
+        <v>368.8</v>
       </c>
       <c r="E7" s="39" t="n">
-        <v>424.21</v>
+        <v>405.02</v>
       </c>
       <c r="F7" s="39" t="n">
-        <v>462.18</v>
+        <v>441.23</v>
       </c>
       <c r="G7" s="39" t="n">
-        <v>500.14</v>
+        <v>477.45</v>
       </c>
     </row>
     <row r="8">
@@ -1884,23 +1884,23 @@
           <t>+10%</t>
         </is>
       </c>
-      <c r="B8" s="39" t="n">
-        <v>334.62</v>
+      <c r="B8" s="38" t="n">
+        <v>319.54</v>
       </c>
       <c r="C8" s="39" t="n">
-        <v>375.62</v>
+        <v>358.65</v>
       </c>
       <c r="D8" s="39" t="n">
-        <v>416.62</v>
+        <v>397.77</v>
       </c>
       <c r="E8" s="39" t="n">
-        <v>457.62</v>
+        <v>436.88</v>
       </c>
       <c r="F8" s="39" t="n">
-        <v>498.62</v>
+        <v>476</v>
       </c>
       <c r="G8" s="39" t="n">
-        <v>539.62</v>
+        <v>515.11</v>
       </c>
     </row>
     <row r="9">
@@ -1910,22 +1910,22 @@
         </is>
       </c>
       <c r="B9" s="39" t="n">
-        <v>358.91</v>
+        <v>342.72</v>
       </c>
       <c r="C9" s="39" t="n">
-        <v>402.95</v>
+        <v>384.73</v>
       </c>
       <c r="D9" s="39" t="n">
-        <v>446.98</v>
+        <v>426.74</v>
       </c>
       <c r="E9" s="39" t="n">
-        <v>491.02</v>
+        <v>468.75</v>
       </c>
       <c r="F9" s="39" t="n">
-        <v>535.0599999999999</v>
+        <v>510.76</v>
       </c>
       <c r="G9" s="39" t="n">
-        <v>579.09</v>
+        <v>552.78</v>
       </c>
     </row>
   </sheetData>
@@ -2388,7 +2388,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HCM $5,929  |  Financials $3,011  |  AI ARR $400  |  Services $719  |  Total $10,059</t>
+          <t>HCM $5,629  |  Financials $2,804  |  AI ARR $400  |  Services $719  |  Total $9,552</t>
         </is>
       </c>
     </row>
@@ -2439,16 +2439,16 @@
         </is>
       </c>
       <c r="B7" s="19" t="n">
-        <v>6581</v>
+        <v>6248</v>
       </c>
       <c r="C7" s="19" t="n">
-        <v>7239</v>
+        <v>6873</v>
       </c>
       <c r="D7" s="19" t="n">
-        <v>7963</v>
+        <v>7560</v>
       </c>
       <c r="E7" s="19" t="n">
-        <v>8680</v>
+        <v>8241</v>
       </c>
     </row>
     <row r="8">
@@ -2458,16 +2458,16 @@
         </is>
       </c>
       <c r="B8" s="19" t="n">
-        <v>3673</v>
+        <v>3421</v>
       </c>
       <c r="C8" s="19" t="n">
-        <v>4408</v>
+        <v>4105</v>
       </c>
       <c r="D8" s="19" t="n">
-        <v>5202</v>
+        <v>4844</v>
       </c>
       <c r="E8" s="19" t="n">
-        <v>6034</v>
+        <v>5619</v>
       </c>
     </row>
     <row r="9">
@@ -2553,16 +2553,16 @@
         </is>
       </c>
       <c r="B13" s="28" t="n">
-        <v>11526</v>
+        <v>10941</v>
       </c>
       <c r="C13" s="28" t="n">
-        <v>13545</v>
+        <v>12876</v>
       </c>
       <c r="D13" s="28" t="n">
-        <v>16006</v>
+        <v>15245</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>18577</v>
+        <v>17723</v>
       </c>
     </row>
     <row r="14">
@@ -2648,16 +2648,16 @@
         </is>
       </c>
       <c r="B18" s="10" t="n">
-        <v>0.7527</v>
+        <v>0.7489</v>
       </c>
       <c r="C18" s="10" t="n">
-        <v>0.7572</v>
+        <v>0.7536</v>
       </c>
       <c r="D18" s="10" t="n">
-        <v>0.7625999999999999</v>
+        <v>0.7592</v>
       </c>
       <c r="E18" s="10" t="n">
-        <v>0.7716</v>
+        <v>0.7685</v>
       </c>
     </row>
     <row r="19">
@@ -2667,16 +2667,16 @@
         </is>
       </c>
       <c r="B19" s="16" t="n">
-        <v>5528</v>
+        <v>5248</v>
       </c>
       <c r="C19" s="16" t="n">
-        <v>6081</v>
+        <v>5773</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>6689</v>
+        <v>6351</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>7291</v>
+        <v>6922</v>
       </c>
     </row>
     <row r="20">
@@ -2686,16 +2686,16 @@
         </is>
       </c>
       <c r="B20" s="16" t="n">
-        <v>2939</v>
+        <v>2737</v>
       </c>
       <c r="C20" s="16" t="n">
-        <v>3571</v>
+        <v>3325</v>
       </c>
       <c r="D20" s="16" t="n">
-        <v>4265</v>
+        <v>3972</v>
       </c>
       <c r="E20" s="16" t="n">
-        <v>5008</v>
+        <v>4664</v>
       </c>
     </row>
     <row r="21">
@@ -2743,16 +2743,16 @@
         </is>
       </c>
       <c r="B23" s="18" t="n">
-        <v>8676</v>
+        <v>8194</v>
       </c>
       <c r="C23" s="18" t="n">
-        <v>10256</v>
+        <v>9703</v>
       </c>
       <c r="D23" s="18" t="n">
-        <v>12205</v>
+        <v>11574</v>
       </c>
       <c r="E23" s="18" t="n">
-        <v>14334</v>
+        <v>13621</v>
       </c>
     </row>
     <row r="25">
@@ -2802,16 +2802,16 @@
         </is>
       </c>
       <c r="B27" s="19" t="n">
-        <v>6285</v>
+        <v>5967</v>
       </c>
       <c r="C27" s="19" t="n">
-        <v>6159</v>
+        <v>5847</v>
       </c>
       <c r="D27" s="19" t="n">
-        <v>5666</v>
+        <v>5380</v>
       </c>
       <c r="E27" s="19" t="n">
-        <v>5100</v>
+        <v>4842</v>
       </c>
     </row>
     <row r="28">
@@ -2821,16 +2821,16 @@
         </is>
       </c>
       <c r="B28" s="19" t="n">
-        <v>3131</v>
+        <v>2916</v>
       </c>
       <c r="C28" s="19" t="n">
-        <v>2944</v>
+        <v>2741</v>
       </c>
       <c r="D28" s="19" t="n">
-        <v>2590</v>
+        <v>2412</v>
       </c>
       <c r="E28" s="19" t="n">
-        <v>2331</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="29">
@@ -2916,16 +2916,16 @@
         </is>
       </c>
       <c r="B33" s="28" t="n">
-        <v>10530</v>
+        <v>9996</v>
       </c>
       <c r="C33" s="28" t="n">
-        <v>10291</v>
+        <v>9777</v>
       </c>
       <c r="D33" s="28" t="n">
-        <v>9471</v>
+        <v>9006</v>
       </c>
       <c r="E33" s="28" t="n">
-        <v>8558</v>
+        <v>8140</v>
       </c>
     </row>
     <row r="34">
@@ -3011,16 +3011,16 @@
         </is>
       </c>
       <c r="B38" s="10" t="n">
-        <v>0.7504</v>
+        <v>0.7465000000000001</v>
       </c>
       <c r="C38" s="10" t="n">
-        <v>0.7516</v>
+        <v>0.7476</v>
       </c>
       <c r="D38" s="10" t="n">
-        <v>0.7507</v>
+        <v>0.7465000000000001</v>
       </c>
       <c r="E38" s="10" t="n">
-        <v>0.7518</v>
+        <v>0.7475000000000001</v>
       </c>
     </row>
     <row r="39">
@@ -3030,16 +3030,16 @@
         </is>
       </c>
       <c r="B39" s="16" t="n">
-        <v>5279</v>
+        <v>5012</v>
       </c>
       <c r="C39" s="16" t="n">
-        <v>5174</v>
+        <v>4912</v>
       </c>
       <c r="D39" s="16" t="n">
-        <v>4760</v>
+        <v>4519</v>
       </c>
       <c r="E39" s="16" t="n">
-        <v>4284</v>
+        <v>4067</v>
       </c>
     </row>
     <row r="40">
@@ -3049,16 +3049,16 @@
         </is>
       </c>
       <c r="B40" s="16" t="n">
-        <v>2505</v>
+        <v>2333</v>
       </c>
       <c r="C40" s="16" t="n">
-        <v>2384</v>
+        <v>2220</v>
       </c>
       <c r="D40" s="16" t="n">
-        <v>2124</v>
+        <v>1978</v>
       </c>
       <c r="E40" s="16" t="n">
-        <v>1935</v>
+        <v>1802</v>
       </c>
     </row>
     <row r="41">
@@ -3106,16 +3106,16 @@
         </is>
       </c>
       <c r="B43" s="18" t="n">
-        <v>7902</v>
+        <v>7462</v>
       </c>
       <c r="C43" s="18" t="n">
-        <v>7735</v>
+        <v>7309</v>
       </c>
       <c r="D43" s="18" t="n">
-        <v>7110</v>
+        <v>6723</v>
       </c>
       <c r="E43" s="18" t="n">
-        <v>6434</v>
+        <v>6085</v>
       </c>
     </row>
     <row r="45">
@@ -3165,16 +3165,16 @@
         </is>
       </c>
       <c r="B47" s="19" t="n">
-        <v>5692</v>
+        <v>5404</v>
       </c>
       <c r="C47" s="19" t="n">
-        <v>5180</v>
+        <v>4917</v>
       </c>
       <c r="D47" s="19" t="n">
-        <v>4662</v>
+        <v>4426</v>
       </c>
       <c r="E47" s="19" t="n">
-        <v>4242</v>
+        <v>4027</v>
       </c>
     </row>
     <row r="48">
@@ -3184,16 +3184,16 @@
         </is>
       </c>
       <c r="B48" s="19" t="n">
-        <v>2830</v>
+        <v>2636</v>
       </c>
       <c r="C48" s="19" t="n">
-        <v>2519</v>
+        <v>2346</v>
       </c>
       <c r="D48" s="19" t="n">
-        <v>2217</v>
+        <v>2064</v>
       </c>
       <c r="E48" s="19" t="n">
-        <v>1973</v>
+        <v>1837</v>
       </c>
     </row>
     <row r="49">
@@ -3279,16 +3279,16 @@
         </is>
       </c>
       <c r="B53" s="28" t="n">
-        <v>9577</v>
+        <v>9095</v>
       </c>
       <c r="C53" s="28" t="n">
-        <v>8760</v>
+        <v>8325</v>
       </c>
       <c r="D53" s="28" t="n">
-        <v>7935</v>
+        <v>7547</v>
       </c>
       <c r="E53" s="28" t="n">
-        <v>7193</v>
+        <v>6843</v>
       </c>
     </row>
     <row r="54">
@@ -3374,16 +3374,16 @@
         </is>
       </c>
       <c r="B58" s="10" t="n">
-        <v>0.7459</v>
+        <v>0.7418</v>
       </c>
       <c r="C58" s="10" t="n">
-        <v>0.7448</v>
+        <v>0.7403999999999999</v>
       </c>
       <c r="D58" s="10" t="n">
-        <v>0.7428</v>
+        <v>0.7382</v>
       </c>
       <c r="E58" s="10" t="n">
-        <v>0.7442</v>
+        <v>0.7395</v>
       </c>
     </row>
     <row r="59">
@@ -3393,16 +3393,16 @@
         </is>
       </c>
       <c r="B59" s="16" t="n">
-        <v>4781</v>
+        <v>4539</v>
       </c>
       <c r="C59" s="16" t="n">
-        <v>4351</v>
+        <v>4131</v>
       </c>
       <c r="D59" s="16" t="n">
-        <v>3916</v>
+        <v>3718</v>
       </c>
       <c r="E59" s="16" t="n">
-        <v>3563</v>
+        <v>3383</v>
       </c>
     </row>
     <row r="60">
@@ -3412,16 +3412,16 @@
         </is>
       </c>
       <c r="B60" s="16" t="n">
-        <v>2264</v>
+        <v>2109</v>
       </c>
       <c r="C60" s="16" t="n">
-        <v>2040</v>
+        <v>1900</v>
       </c>
       <c r="D60" s="16" t="n">
-        <v>1818</v>
+        <v>1693</v>
       </c>
       <c r="E60" s="16" t="n">
-        <v>1637</v>
+        <v>1525</v>
       </c>
     </row>
     <row r="61">
@@ -3469,16 +3469,16 @@
         </is>
       </c>
       <c r="B63" s="18" t="n">
-        <v>7144</v>
+        <v>6746</v>
       </c>
       <c r="C63" s="18" t="n">
-        <v>6524</v>
+        <v>6164</v>
       </c>
       <c r="D63" s="18" t="n">
-        <v>5894</v>
+        <v>5571</v>
       </c>
       <c r="E63" s="18" t="n">
-        <v>5354</v>
+        <v>5061</v>
       </c>
     </row>
   </sheetData>
@@ -4070,19 +4070,19 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>5929</v>
+        <v>5629</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>6581</v>
+        <v>6248</v>
       </c>
       <c r="D6" s="27" t="n">
-        <v>7239</v>
+        <v>6873</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>7963</v>
+        <v>7560</v>
       </c>
       <c r="F6" s="27" t="n">
-        <v>8680</v>
+        <v>8241</v>
       </c>
     </row>
     <row r="7">
@@ -4092,19 +4092,19 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>3011</v>
+        <v>2804</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>3673</v>
+        <v>3421</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>4408</v>
+        <v>4105</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>5202</v>
+        <v>4844</v>
       </c>
       <c r="F7" s="27" t="n">
-        <v>6034</v>
+        <v>5619</v>
       </c>
     </row>
     <row r="8">
@@ -4161,16 +4161,16 @@
         <v>9552</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>11526</v>
+        <v>10941</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>13545</v>
+        <v>12876</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>16006</v>
+        <v>15245</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>18577</v>
+        <v>17723</v>
       </c>
     </row>
     <row r="11">
@@ -4183,16 +4183,16 @@
         <v>2624</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>2850</v>
+        <v>2747</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>3289</v>
+        <v>3173</v>
       </c>
       <c r="E11" s="27" t="n">
-        <v>3801</v>
+        <v>3671</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>4243</v>
+        <v>4102</v>
       </c>
     </row>
     <row r="12">
@@ -4205,16 +4205,16 @@
         <v>6928</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>8676</v>
+        <v>8194</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>10256</v>
+        <v>9703</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>12205</v>
+        <v>11574</v>
       </c>
       <c r="F12" s="18" t="n">
-        <v>14334</v>
+        <v>13621</v>
       </c>
     </row>
     <row r="13">
@@ -4227,16 +4227,16 @@
         <v>2679</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>2997</v>
+        <v>2845</v>
       </c>
       <c r="D13" s="27" t="n">
-        <v>3386</v>
+        <v>3219</v>
       </c>
       <c r="E13" s="27" t="n">
-        <v>3841</v>
+        <v>3659</v>
       </c>
       <c r="F13" s="27" t="n">
-        <v>4273</v>
+        <v>4076</v>
       </c>
     </row>
     <row r="14">
@@ -4249,16 +4249,16 @@
         <v>2616</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>2882</v>
+        <v>2735</v>
       </c>
       <c r="D14" s="27" t="n">
-        <v>3115</v>
+        <v>2961</v>
       </c>
       <c r="E14" s="27" t="n">
-        <v>3361</v>
+        <v>3201</v>
       </c>
       <c r="F14" s="27" t="n">
-        <v>3715</v>
+        <v>3545</v>
       </c>
     </row>
     <row r="15">
@@ -4271,16 +4271,16 @@
         <v>912</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>1037</v>
+        <v>985</v>
       </c>
       <c r="D15" s="27" t="n">
-        <v>1151</v>
+        <v>1094</v>
       </c>
       <c r="E15" s="27" t="n">
-        <v>1280</v>
+        <v>1220</v>
       </c>
       <c r="F15" s="27" t="n">
-        <v>1486</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="16">
@@ -4293,16 +4293,16 @@
         <v>721</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1422</v>
+        <v>1309</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>2206</v>
+        <v>2050</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>3253</v>
+        <v>3047</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>4315</v>
+        <v>4062</v>
       </c>
     </row>
     <row r="17">
@@ -4315,16 +4315,16 @@
         <v>0.07548157453936348</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>0.1234</v>
+        <v>0.1196</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>0.1629</v>
+        <v>0.1593</v>
       </c>
       <c r="E17" s="25" t="n">
-        <v>0.2033</v>
+        <v>0.1999</v>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.2323</v>
+        <v>0.2292</v>
       </c>
     </row>
     <row r="18">
@@ -4340,13 +4340,13 @@
         <v>218</v>
       </c>
       <c r="D18" s="26" t="n">
-        <v>333</v>
+        <v>326</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>445</v>
+        <v>428</v>
       </c>
       <c r="F18" s="26" t="n">
-        <v>537</v>
+        <v>511</v>
       </c>
     </row>
     <row r="19">
@@ -4381,16 +4381,16 @@
         <v>1009</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1535</v>
+        <v>1422</v>
       </c>
       <c r="D20" s="27" t="n">
-        <v>2434</v>
+        <v>2272</v>
       </c>
       <c r="E20" s="27" t="n">
-        <v>3593</v>
+        <v>3371</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>4748</v>
+        <v>4468</v>
       </c>
     </row>
     <row r="21">
@@ -4403,16 +4403,16 @@
         <v>-316</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>-384</v>
+        <v>-355</v>
       </c>
       <c r="D21" s="27" t="n">
-        <v>-609</v>
+        <v>-568</v>
       </c>
       <c r="E21" s="27" t="n">
-        <v>-898</v>
+        <v>-843</v>
       </c>
       <c r="F21" s="27" t="n">
-        <v>-1187</v>
+        <v>-1117</v>
       </c>
     </row>
     <row r="22">
@@ -4425,16 +4425,16 @@
         <v>693</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>1151</v>
+        <v>1066</v>
       </c>
       <c r="D22" s="18" t="n">
-        <v>1826</v>
+        <v>1704</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>2695</v>
+        <v>2528</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>3561</v>
+        <v>3351</v>
       </c>
     </row>
     <row r="23">
@@ -4469,16 +4469,16 @@
         <v>2.59</v>
       </c>
       <c r="C24" s="32" t="n">
-        <v>4.38</v>
+        <v>4.06</v>
       </c>
       <c r="D24" s="32" t="n">
-        <v>7.09</v>
+        <v>6.62</v>
       </c>
       <c r="E24" s="32" t="n">
-        <v>10.74</v>
+        <v>10.07</v>
       </c>
       <c r="F24" s="32" t="n">
-        <v>14.55</v>
+        <v>13.7</v>
       </c>
     </row>
     <row r="26">
@@ -4515,16 +4515,16 @@
         <v>1501</v>
       </c>
       <c r="C28" s="27" t="n">
-        <v>4235</v>
+        <v>3911</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>7032</v>
+        <v>6489</v>
       </c>
       <c r="E28" s="27" t="n">
-        <v>9260</v>
+        <v>8448</v>
       </c>
       <c r="F28" s="27" t="n">
-        <v>11264</v>
+        <v>10139</v>
       </c>
     </row>
     <row r="29">
@@ -4559,16 +4559,16 @@
         <v>2332</v>
       </c>
       <c r="C30" s="27" t="n">
-        <v>2814</v>
+        <v>2671</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>3307</v>
+        <v>3144</v>
       </c>
       <c r="E30" s="27" t="n">
-        <v>3908</v>
+        <v>3722</v>
       </c>
       <c r="F30" s="27" t="n">
-        <v>4535</v>
+        <v>4327</v>
       </c>
     </row>
     <row r="31">
@@ -4581,16 +4581,16 @@
         <v>348</v>
       </c>
       <c r="C31" s="27" t="n">
-        <v>415</v>
+        <v>394</v>
       </c>
       <c r="D31" s="27" t="n">
-        <v>488</v>
+        <v>464</v>
       </c>
       <c r="E31" s="27" t="n">
-        <v>576</v>
+        <v>549</v>
       </c>
       <c r="F31" s="27" t="n">
-        <v>669</v>
+        <v>638</v>
       </c>
     </row>
     <row r="32">
@@ -4603,16 +4603,16 @@
         <v>306</v>
       </c>
       <c r="C32" s="27" t="n">
-        <v>369</v>
+        <v>350</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>433</v>
+        <v>412</v>
       </c>
       <c r="E32" s="27" t="n">
-        <v>512</v>
+        <v>488</v>
       </c>
       <c r="F32" s="27" t="n">
-        <v>594</v>
+        <v>567</v>
       </c>
     </row>
     <row r="33">
@@ -4625,16 +4625,16 @@
         <v>1093</v>
       </c>
       <c r="C33" s="27" t="n">
-        <v>1087</v>
+        <v>1075</v>
       </c>
       <c r="D33" s="27" t="n">
-        <v>1106</v>
+        <v>1081</v>
       </c>
       <c r="E33" s="27" t="n">
-        <v>1159</v>
+        <v>1119</v>
       </c>
       <c r="F33" s="27" t="n">
-        <v>1249</v>
+        <v>1191</v>
       </c>
     </row>
     <row r="34">
@@ -4713,16 +4713,16 @@
         <v>634</v>
       </c>
       <c r="C37" s="27" t="n">
-        <v>761</v>
+        <v>722</v>
       </c>
       <c r="D37" s="27" t="n">
-        <v>894</v>
+        <v>850</v>
       </c>
       <c r="E37" s="27" t="n">
-        <v>1056</v>
+        <v>1006</v>
       </c>
       <c r="F37" s="27" t="n">
-        <v>1226</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="38">
@@ -4779,16 +4779,16 @@
         <v>18074</v>
       </c>
       <c r="C40" s="18" t="n">
-        <v>21441</v>
+        <v>20883</v>
       </c>
       <c r="D40" s="18" t="n">
-        <v>24920</v>
+        <v>24099</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>28031</v>
+        <v>26891</v>
       </c>
       <c r="F40" s="18" t="n">
-        <v>30997</v>
+        <v>29492</v>
       </c>
     </row>
     <row r="42">
@@ -4813,16 +4813,16 @@
         <v>142</v>
       </c>
       <c r="C43" s="27" t="n">
-        <v>173</v>
+        <v>164</v>
       </c>
       <c r="D43" s="27" t="n">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="E43" s="27" t="n">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="F43" s="27" t="n">
-        <v>279</v>
+        <v>266</v>
       </c>
     </row>
     <row r="44">
@@ -4835,16 +4835,16 @@
         <v>642</v>
       </c>
       <c r="C44" s="27" t="n">
-        <v>784</v>
+        <v>744</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>921</v>
+        <v>876</v>
       </c>
       <c r="E44" s="27" t="n">
-        <v>1088</v>
+        <v>1037</v>
       </c>
       <c r="F44" s="27" t="n">
-        <v>1263</v>
+        <v>1205</v>
       </c>
     </row>
     <row r="45">
@@ -4857,16 +4857,16 @@
         <v>454</v>
       </c>
       <c r="C45" s="27" t="n">
-        <v>553</v>
+        <v>525</v>
       </c>
       <c r="D45" s="27" t="n">
-        <v>650</v>
+        <v>618</v>
       </c>
       <c r="E45" s="27" t="n">
-        <v>768</v>
+        <v>732</v>
       </c>
       <c r="F45" s="27" t="n">
-        <v>892</v>
+        <v>851</v>
       </c>
     </row>
     <row r="46">
@@ -4879,16 +4879,16 @@
         <v>5010</v>
       </c>
       <c r="C46" s="27" t="n">
-        <v>5918</v>
+        <v>5610</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>7225</v>
+        <v>6873</v>
       </c>
       <c r="E46" s="27" t="n">
-        <v>8678</v>
+        <v>8278</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>10094</v>
+        <v>9645</v>
       </c>
     </row>
     <row r="47">
@@ -5011,16 +5011,16 @@
         <v>10269</v>
       </c>
       <c r="C52" s="18" t="n">
-        <v>11449</v>
+        <v>11064</v>
       </c>
       <c r="D52" s="18" t="n">
-        <v>13020</v>
+        <v>12581</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>14795</v>
+        <v>14296</v>
       </c>
       <c r="F52" s="18" t="n">
-        <v>16548</v>
+        <v>15988</v>
       </c>
     </row>
     <row r="54">
@@ -5045,16 +5045,16 @@
         <v>12673</v>
       </c>
       <c r="C55" s="27" t="n">
-        <v>14402</v>
+        <v>14314</v>
       </c>
       <c r="D55" s="27" t="n">
-        <v>16163</v>
+        <v>15988</v>
       </c>
       <c r="E55" s="27" t="n">
-        <v>18084</v>
+        <v>17817</v>
       </c>
       <c r="F55" s="27" t="n">
-        <v>20128</v>
+        <v>19767</v>
       </c>
     </row>
     <row r="56">
@@ -5089,16 +5089,16 @@
         <v>-512</v>
       </c>
       <c r="C57" s="27" t="n">
-        <v>639</v>
+        <v>554</v>
       </c>
       <c r="D57" s="27" t="n">
-        <v>2465</v>
+        <v>2258</v>
       </c>
       <c r="E57" s="27" t="n">
-        <v>5160</v>
+        <v>4786</v>
       </c>
       <c r="F57" s="27" t="n">
-        <v>8721</v>
+        <v>8137</v>
       </c>
     </row>
     <row r="58">
@@ -5133,16 +5133,16 @@
         <v>7805</v>
       </c>
       <c r="C59" s="18" t="n">
-        <v>9992</v>
+        <v>9819</v>
       </c>
       <c r="D59" s="18" t="n">
-        <v>11900</v>
+        <v>11518</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>13236</v>
+        <v>12595</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>14449</v>
+        <v>13504</v>
       </c>
     </row>
     <row r="61">
@@ -5155,16 +5155,16 @@
         <v>0</v>
       </c>
       <c r="C61" s="41" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="D61" s="41" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="E61" s="41" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="F61" s="41" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
     </row>
     <row r="63">
@@ -5201,16 +5201,16 @@
         <v>693</v>
       </c>
       <c r="C65" s="27" t="n">
-        <v>1151</v>
+        <v>1066</v>
       </c>
       <c r="D65" s="27" t="n">
-        <v>1826</v>
+        <v>1704</v>
       </c>
       <c r="E65" s="27" t="n">
-        <v>2695</v>
+        <v>2528</v>
       </c>
       <c r="F65" s="27" t="n">
-        <v>3561</v>
+        <v>3351</v>
       </c>
     </row>
     <row r="66">
@@ -5267,16 +5267,16 @@
         <v>1626</v>
       </c>
       <c r="C68" s="27" t="n">
-        <v>1729</v>
+        <v>1641</v>
       </c>
       <c r="D68" s="27" t="n">
-        <v>1761</v>
+        <v>1674</v>
       </c>
       <c r="E68" s="27" t="n">
-        <v>1921</v>
+        <v>1829</v>
       </c>
       <c r="F68" s="27" t="n">
-        <v>2044</v>
+        <v>1950</v>
       </c>
     </row>
     <row r="69">
@@ -5287,16 +5287,16 @@
       </c>
       <c r="B69" s="40" t="n"/>
       <c r="C69" s="42" t="n">
-        <v>-482</v>
+        <v>-339</v>
       </c>
       <c r="D69" s="42" t="n">
-        <v>-493</v>
+        <v>-472</v>
       </c>
       <c r="E69" s="42" t="n">
-        <v>-601</v>
+        <v>-578</v>
       </c>
       <c r="F69" s="42" t="n">
-        <v>-628</v>
+        <v>-605</v>
       </c>
     </row>
     <row r="70">
@@ -5307,16 +5307,16 @@
       </c>
       <c r="B70" s="40" t="n"/>
       <c r="C70" s="42" t="n">
-        <v>908</v>
+        <v>600</v>
       </c>
       <c r="D70" s="42" t="n">
-        <v>1307</v>
+        <v>1263</v>
       </c>
       <c r="E70" s="42" t="n">
-        <v>1453</v>
+        <v>1405</v>
       </c>
       <c r="F70" s="42" t="n">
-        <v>1416</v>
+        <v>1367</v>
       </c>
     </row>
     <row r="71">
@@ -5327,16 +5327,16 @@
       </c>
       <c r="B71" s="40" t="n"/>
       <c r="C71" s="42" t="n">
-        <v>142</v>
+        <v>102</v>
       </c>
       <c r="D71" s="42" t="n">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E71" s="42" t="n">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="F71" s="42" t="n">
-        <v>175</v>
+        <v>169</v>
       </c>
     </row>
     <row r="72">
@@ -5347,16 +5347,16 @@
       </c>
       <c r="B72" s="40" t="n"/>
       <c r="C72" s="42" t="n">
-        <v>130</v>
+        <v>93</v>
       </c>
       <c r="D72" s="42" t="n">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="E72" s="42" t="n">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="F72" s="42" t="n">
-        <v>162</v>
+        <v>156</v>
       </c>
     </row>
     <row r="73">
@@ -5367,16 +5367,16 @@
       </c>
       <c r="B73" s="40" t="n"/>
       <c r="C73" s="42" t="n">
-        <v>-67</v>
+        <v>-46</v>
       </c>
       <c r="D73" s="42" t="n">
-        <v>-73</v>
+        <v>-70</v>
       </c>
       <c r="E73" s="42" t="n">
+        <v>-85</v>
+      </c>
+      <c r="F73" s="42" t="n">
         <v>-89</v>
-      </c>
-      <c r="F73" s="42" t="n">
-        <v>-93</v>
       </c>
     </row>
     <row r="74">
@@ -5387,16 +5387,16 @@
       </c>
       <c r="B74" s="40" t="n"/>
       <c r="C74" s="42" t="n">
+        <v>-132</v>
+      </c>
+      <c r="D74" s="42" t="n">
         <v>-190</v>
       </c>
-      <c r="D74" s="42" t="n">
-        <v>-198</v>
-      </c>
       <c r="E74" s="42" t="n">
-        <v>-241</v>
+        <v>-232</v>
       </c>
       <c r="F74" s="42" t="n">
-        <v>-252</v>
+        <v>-243</v>
       </c>
     </row>
     <row r="75">
@@ -5408,16 +5408,16 @@
         <v>2939</v>
       </c>
       <c r="C75" s="18" t="n">
-        <v>3658</v>
+        <v>3322</v>
       </c>
       <c r="D75" s="18" t="n">
-        <v>4747</v>
+        <v>4515</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>5828</v>
+        <v>5543</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>6768</v>
+        <v>6438</v>
       </c>
     </row>
     <row r="77">
@@ -5442,16 +5442,16 @@
         <v>-162</v>
       </c>
       <c r="C78" s="27" t="n">
-        <v>-231</v>
+        <v>-219</v>
       </c>
       <c r="D78" s="27" t="n">
-        <v>-271</v>
+        <v>-258</v>
       </c>
       <c r="E78" s="27" t="n">
-        <v>-320</v>
+        <v>-305</v>
       </c>
       <c r="F78" s="27" t="n">
-        <v>-372</v>
+        <v>-354</v>
       </c>
     </row>
     <row r="79">
@@ -5503,16 +5503,16 @@
         <v>-162</v>
       </c>
       <c r="C81" s="18" t="n">
-        <v>-231</v>
+        <v>-219</v>
       </c>
       <c r="D81" s="18" t="n">
-        <v>-271</v>
+        <v>-258</v>
       </c>
       <c r="E81" s="18" t="n">
-        <v>-320</v>
+        <v>-305</v>
       </c>
       <c r="F81" s="18" t="n">
-        <v>-372</v>
+        <v>-354</v>
       </c>
     </row>
     <row r="83">
@@ -5614,16 +5614,16 @@
       </c>
       <c r="B89" s="16" t="n"/>
       <c r="C89" s="27" t="n">
-        <v>2734</v>
+        <v>2410</v>
       </c>
       <c r="D89" s="27" t="n">
-        <v>2797</v>
+        <v>2578</v>
       </c>
       <c r="E89" s="27" t="n">
-        <v>2228</v>
+        <v>1958</v>
       </c>
       <c r="F89" s="27" t="n">
-        <v>2004</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="90">
@@ -5639,13 +5639,13 @@
         <v>1501</v>
       </c>
       <c r="D90" s="27" t="n">
-        <v>4235</v>
+        <v>3911</v>
       </c>
       <c r="E90" s="27" t="n">
-        <v>7032</v>
+        <v>6489</v>
       </c>
       <c r="F90" s="27" t="n">
-        <v>9260</v>
+        <v>8448</v>
       </c>
     </row>
     <row r="91">
@@ -5658,16 +5658,16 @@
         <v>1501</v>
       </c>
       <c r="C91" s="18" t="n">
-        <v>4235</v>
+        <v>3911</v>
       </c>
       <c r="D91" s="18" t="n">
-        <v>7032</v>
+        <v>6489</v>
       </c>
       <c r="E91" s="18" t="n">
-        <v>9260</v>
+        <v>8448</v>
       </c>
       <c r="F91" s="18" t="n">
-        <v>11264</v>
+        <v>10139</v>
       </c>
     </row>
     <row r="93">
@@ -5830,19 +5830,19 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>5929</v>
+        <v>5629</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>6285</v>
+        <v>5967</v>
       </c>
       <c r="D6" s="27" t="n">
-        <v>6159</v>
+        <v>5847</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>5666</v>
+        <v>5380</v>
       </c>
       <c r="F6" s="27" t="n">
-        <v>5100</v>
+        <v>4842</v>
       </c>
     </row>
     <row r="7">
@@ -5852,19 +5852,19 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>3011</v>
+        <v>2804</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>3131</v>
+        <v>2916</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>2944</v>
+        <v>2741</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>2590</v>
+        <v>2412</v>
       </c>
       <c r="F7" s="27" t="n">
-        <v>2331</v>
+        <v>2171</v>
       </c>
     </row>
     <row r="8">
@@ -5921,16 +5921,16 @@
         <v>9552</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>10530</v>
+        <v>9996</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>10291</v>
+        <v>9777</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>9471</v>
+        <v>9006</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>8558</v>
+        <v>8140</v>
       </c>
     </row>
     <row r="11">
@@ -5943,16 +5943,16 @@
         <v>2624</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>2628</v>
+        <v>2534</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>2556</v>
+        <v>2468</v>
       </c>
       <c r="E11" s="27" t="n">
-        <v>2361</v>
+        <v>2283</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>2124</v>
+        <v>2055</v>
       </c>
     </row>
     <row r="12">
@@ -5965,16 +5965,16 @@
         <v>6928</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>7902</v>
+        <v>7462</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>7735</v>
+        <v>7309</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>7110</v>
+        <v>6723</v>
       </c>
       <c r="F12" s="18" t="n">
-        <v>6434</v>
+        <v>6085</v>
       </c>
     </row>
     <row r="13">
@@ -5987,16 +5987,16 @@
         <v>2679</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>2527</v>
+        <v>2399</v>
       </c>
       <c r="D13" s="27" t="n">
-        <v>2058</v>
+        <v>1955</v>
       </c>
       <c r="E13" s="27" t="n">
-        <v>1515</v>
+        <v>1441</v>
       </c>
       <c r="F13" s="27" t="n">
-        <v>1113</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="14">
@@ -6009,16 +6009,16 @@
         <v>2616</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>2317</v>
+        <v>2199</v>
       </c>
       <c r="D14" s="27" t="n">
-        <v>1749</v>
+        <v>1662</v>
       </c>
       <c r="E14" s="27" t="n">
-        <v>1231</v>
+        <v>1171</v>
       </c>
       <c r="F14" s="27" t="n">
-        <v>856</v>
+        <v>814</v>
       </c>
     </row>
     <row r="15">
@@ -6031,16 +6031,16 @@
         <v>912</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>842</v>
+        <v>800</v>
       </c>
       <c r="D15" s="27" t="n">
-        <v>720</v>
+        <v>684</v>
       </c>
       <c r="E15" s="27" t="n">
-        <v>568</v>
+        <v>540</v>
       </c>
       <c r="F15" s="27" t="n">
-        <v>428</v>
+        <v>407</v>
       </c>
     </row>
     <row r="16">
@@ -6053,16 +6053,16 @@
         <v>721</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1907</v>
+        <v>1771</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>2905</v>
+        <v>2721</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>3517</v>
+        <v>3307</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>3787</v>
+        <v>3567</v>
       </c>
     </row>
     <row r="17">
@@ -6075,16 +6075,16 @@
         <v>0.07548157453936348</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>0.1811</v>
+        <v>0.1772</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>0.2823</v>
+        <v>0.2783</v>
       </c>
       <c r="E17" s="25" t="n">
-        <v>0.3714</v>
+        <v>0.3672</v>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.4425</v>
+        <v>0.4382</v>
       </c>
     </row>
     <row r="18">
@@ -6100,13 +6100,13 @@
         <v>218</v>
       </c>
       <c r="D18" s="26" t="n">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="F18" s="26" t="n">
-        <v>226</v>
+        <v>212</v>
       </c>
     </row>
     <row r="19">
@@ -6141,16 +6141,16 @@
         <v>1009</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>2020</v>
+        <v>1885</v>
       </c>
       <c r="D20" s="27" t="n">
-        <v>3080</v>
+        <v>2890</v>
       </c>
       <c r="E20" s="27" t="n">
-        <v>3689</v>
+        <v>3468</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>3909</v>
+        <v>3675</v>
       </c>
     </row>
     <row r="21">
@@ -6163,16 +6163,16 @@
         <v>-316</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>-505</v>
+        <v>-471</v>
       </c>
       <c r="D21" s="27" t="n">
-        <v>-770</v>
+        <v>-722</v>
       </c>
       <c r="E21" s="27" t="n">
-        <v>-922</v>
+        <v>-867</v>
       </c>
       <c r="F21" s="27" t="n">
-        <v>-977</v>
+        <v>-919</v>
       </c>
     </row>
     <row r="22">
@@ -6185,16 +6185,16 @@
         <v>693</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>1515</v>
+        <v>1413</v>
       </c>
       <c r="D22" s="18" t="n">
-        <v>2310</v>
+        <v>2167</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>2767</v>
+        <v>2601</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>2931</v>
+        <v>2756</v>
       </c>
     </row>
     <row r="23">
@@ -6229,16 +6229,16 @@
         <v>2.59</v>
       </c>
       <c r="C24" s="32" t="n">
-        <v>5.89</v>
+        <v>5.49</v>
       </c>
       <c r="D24" s="32" t="n">
-        <v>9.66</v>
+        <v>9.06</v>
       </c>
       <c r="E24" s="32" t="n">
-        <v>12.71</v>
+        <v>11.95</v>
       </c>
       <c r="F24" s="32" t="n">
-        <v>14.96</v>
+        <v>14.06</v>
       </c>
     </row>
     <row r="26">
@@ -6275,16 +6275,16 @@
         <v>1501</v>
       </c>
       <c r="C28" s="27" t="n">
-        <v>2833</v>
+        <v>2542</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>2636</v>
+        <v>2232</v>
       </c>
       <c r="E28" s="27" t="n">
-        <v>1450</v>
+        <v>954</v>
       </c>
       <c r="F28" s="27" t="n">
-        <v>119</v>
+        <v>-467</v>
       </c>
     </row>
     <row r="29">
@@ -6319,16 +6319,16 @@
         <v>2332</v>
       </c>
       <c r="C30" s="27" t="n">
-        <v>2571</v>
+        <v>2440</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>2512</v>
+        <v>2387</v>
       </c>
       <c r="E30" s="27" t="n">
-        <v>2312</v>
+        <v>2199</v>
       </c>
       <c r="F30" s="27" t="n">
-        <v>2089</v>
+        <v>1987</v>
       </c>
     </row>
     <row r="31">
@@ -6341,16 +6341,16 @@
         <v>348</v>
       </c>
       <c r="C31" s="27" t="n">
-        <v>379</v>
+        <v>360</v>
       </c>
       <c r="D31" s="27" t="n">
-        <v>370</v>
+        <v>352</v>
       </c>
       <c r="E31" s="27" t="n">
-        <v>341</v>
+        <v>324</v>
       </c>
       <c r="F31" s="27" t="n">
-        <v>308</v>
+        <v>293</v>
       </c>
     </row>
     <row r="32">
@@ -6363,16 +6363,16 @@
         <v>306</v>
       </c>
       <c r="C32" s="27" t="n">
-        <v>337</v>
+        <v>320</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>329</v>
+        <v>313</v>
       </c>
       <c r="E32" s="27" t="n">
-        <v>303</v>
+        <v>288</v>
       </c>
       <c r="F32" s="27" t="n">
-        <v>274</v>
+        <v>260</v>
       </c>
     </row>
     <row r="33">
@@ -6385,16 +6385,16 @@
         <v>1093</v>
       </c>
       <c r="C33" s="27" t="n">
-        <v>1067</v>
+        <v>1056</v>
       </c>
       <c r="D33" s="27" t="n">
-        <v>1021</v>
+        <v>1000</v>
       </c>
       <c r="E33" s="27" t="n">
-        <v>943</v>
+        <v>913</v>
       </c>
       <c r="F33" s="27" t="n">
-        <v>832</v>
+        <v>794</v>
       </c>
     </row>
     <row r="34">
@@ -6473,16 +6473,16 @@
         <v>634</v>
       </c>
       <c r="C37" s="27" t="n">
-        <v>695</v>
+        <v>660</v>
       </c>
       <c r="D37" s="27" t="n">
-        <v>679</v>
+        <v>645</v>
       </c>
       <c r="E37" s="27" t="n">
-        <v>625</v>
+        <v>594</v>
       </c>
       <c r="F37" s="27" t="n">
-        <v>565</v>
+        <v>537</v>
       </c>
     </row>
     <row r="38">
@@ -6539,16 +6539,16 @@
         <v>18074</v>
       </c>
       <c r="C40" s="18" t="n">
-        <v>19642</v>
+        <v>19137</v>
       </c>
       <c r="D40" s="18" t="n">
-        <v>19208</v>
+        <v>18589</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>17534</v>
+        <v>16832</v>
       </c>
       <c r="F40" s="18" t="n">
-        <v>15647</v>
+        <v>14865</v>
       </c>
     </row>
     <row r="42">
@@ -6573,16 +6573,16 @@
         <v>142</v>
       </c>
       <c r="C43" s="27" t="n">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="D43" s="27" t="n">
-        <v>154</v>
+        <v>147</v>
       </c>
       <c r="E43" s="27" t="n">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="F43" s="27" t="n">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44">
@@ -6595,16 +6595,16 @@
         <v>642</v>
       </c>
       <c r="C44" s="27" t="n">
-        <v>716</v>
+        <v>680</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>700</v>
+        <v>665</v>
       </c>
       <c r="E44" s="27" t="n">
-        <v>644</v>
+        <v>612</v>
       </c>
       <c r="F44" s="27" t="n">
-        <v>582</v>
+        <v>554</v>
       </c>
     </row>
     <row r="45">
@@ -6617,16 +6617,16 @@
         <v>454</v>
       </c>
       <c r="C45" s="27" t="n">
-        <v>505</v>
+        <v>480</v>
       </c>
       <c r="D45" s="27" t="n">
-        <v>494</v>
+        <v>469</v>
       </c>
       <c r="E45" s="27" t="n">
-        <v>455</v>
+        <v>432</v>
       </c>
       <c r="F45" s="27" t="n">
-        <v>411</v>
+        <v>391</v>
       </c>
     </row>
     <row r="46">
@@ -6639,16 +6639,16 @@
         <v>5010</v>
       </c>
       <c r="C46" s="27" t="n">
-        <v>5266</v>
+        <v>4986</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>5215</v>
+        <v>4945</v>
       </c>
       <c r="E46" s="27" t="n">
-        <v>4790</v>
+        <v>4546</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>4332</v>
+        <v>4112</v>
       </c>
     </row>
     <row r="47">
@@ -6771,16 +6771,16 @@
         <v>10269</v>
       </c>
       <c r="C52" s="18" t="n">
-        <v>10666</v>
+        <v>10316</v>
       </c>
       <c r="D52" s="18" t="n">
-        <v>10584</v>
+        <v>10247</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>10052</v>
+        <v>9747</v>
       </c>
       <c r="F52" s="18" t="n">
-        <v>9474</v>
+        <v>9200</v>
       </c>
     </row>
     <row r="54">
@@ -6805,16 +6805,16 @@
         <v>12673</v>
       </c>
       <c r="C55" s="27" t="n">
-        <v>14042</v>
+        <v>13973</v>
       </c>
       <c r="D55" s="27" t="n">
-        <v>14968</v>
+        <v>14853</v>
       </c>
       <c r="E55" s="27" t="n">
-        <v>15536</v>
+        <v>15393</v>
       </c>
       <c r="F55" s="27" t="n">
-        <v>15878</v>
+        <v>15719</v>
       </c>
     </row>
     <row r="56">
@@ -6849,16 +6849,16 @@
         <v>-512</v>
       </c>
       <c r="C57" s="27" t="n">
-        <v>677</v>
+        <v>591</v>
       </c>
       <c r="D57" s="27" t="n">
-        <v>1762</v>
+        <v>1595</v>
       </c>
       <c r="E57" s="27" t="n">
-        <v>2919</v>
+        <v>2665</v>
       </c>
       <c r="F57" s="27" t="n">
-        <v>4207</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="58">
@@ -6893,16 +6893,16 @@
         <v>7805</v>
       </c>
       <c r="C59" s="18" t="n">
-        <v>8976</v>
+        <v>8821</v>
       </c>
       <c r="D59" s="18" t="n">
-        <v>8624</v>
+        <v>8342</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>7482</v>
+        <v>7085</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>6173</v>
+        <v>5665</v>
       </c>
     </row>
     <row r="61">
@@ -6921,10 +6921,10 @@
         <v>-0</v>
       </c>
       <c r="E61" s="41" t="n">
+        <v>-0</v>
+      </c>
+      <c r="F61" s="41" t="n">
         <v>0</v>
-      </c>
-      <c r="F61" s="41" t="n">
-        <v>-0</v>
       </c>
     </row>
     <row r="63">
@@ -6961,16 +6961,16 @@
         <v>693</v>
       </c>
       <c r="C65" s="27" t="n">
-        <v>1515</v>
+        <v>1413</v>
       </c>
       <c r="D65" s="27" t="n">
-        <v>2310</v>
+        <v>2167</v>
       </c>
       <c r="E65" s="27" t="n">
-        <v>2767</v>
+        <v>2601</v>
       </c>
       <c r="F65" s="27" t="n">
-        <v>2931</v>
+        <v>2756</v>
       </c>
     </row>
     <row r="66">
@@ -7027,16 +7027,16 @@
         <v>1626</v>
       </c>
       <c r="C68" s="27" t="n">
-        <v>1369</v>
+        <v>1300</v>
       </c>
       <c r="D68" s="27" t="n">
-        <v>926</v>
+        <v>880</v>
       </c>
       <c r="E68" s="27" t="n">
-        <v>568</v>
+        <v>540</v>
       </c>
       <c r="F68" s="27" t="n">
-        <v>342</v>
+        <v>326</v>
       </c>
     </row>
     <row r="69">
@@ -7047,16 +7047,16 @@
       </c>
       <c r="B69" s="40" t="n"/>
       <c r="C69" s="42" t="n">
-        <v>-239</v>
+        <v>-108</v>
       </c>
       <c r="D69" s="42" t="n">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="E69" s="42" t="n">
-        <v>200</v>
+        <v>188</v>
       </c>
       <c r="F69" s="42" t="n">
-        <v>223</v>
+        <v>211</v>
       </c>
     </row>
     <row r="70">
@@ -7067,16 +7067,16 @@
       </c>
       <c r="B70" s="40" t="n"/>
       <c r="C70" s="42" t="n">
-        <v>256</v>
+        <v>-24</v>
       </c>
       <c r="D70" s="42" t="n">
-        <v>-51</v>
+        <v>-41</v>
       </c>
       <c r="E70" s="42" t="n">
-        <v>-425</v>
+        <v>-399</v>
       </c>
       <c r="F70" s="42" t="n">
-        <v>-459</v>
+        <v>-434</v>
       </c>
     </row>
     <row r="71">
@@ -7087,16 +7087,16 @@
       </c>
       <c r="B71" s="40" t="n"/>
       <c r="C71" s="42" t="n">
-        <v>74</v>
+        <v>38</v>
       </c>
       <c r="D71" s="42" t="n">
-        <v>-16</v>
+        <v>-15</v>
       </c>
       <c r="E71" s="42" t="n">
-        <v>-56</v>
+        <v>-52</v>
       </c>
       <c r="F71" s="42" t="n">
-        <v>-62</v>
+        <v>-59</v>
       </c>
     </row>
     <row r="72">
@@ -7107,16 +7107,16 @@
       </c>
       <c r="B72" s="40" t="n"/>
       <c r="C72" s="42" t="n">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="D72" s="42" t="n">
-        <v>-15</v>
+        <v>-14</v>
       </c>
       <c r="E72" s="42" t="n">
-        <v>-52</v>
+        <v>-49</v>
       </c>
       <c r="F72" s="42" t="n">
-        <v>-58</v>
+        <v>-55</v>
       </c>
     </row>
     <row r="73">
@@ -7127,16 +7127,16 @@
       </c>
       <c r="B73" s="40" t="n"/>
       <c r="C73" s="42" t="n">
-        <v>-31</v>
+        <v>-12</v>
       </c>
       <c r="D73" s="42" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E73" s="42" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F73" s="42" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="74">
@@ -7147,16 +7147,16 @@
       </c>
       <c r="B74" s="40" t="n"/>
       <c r="C74" s="42" t="n">
-        <v>-92</v>
+        <v>-40</v>
       </c>
       <c r="D74" s="42" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="E74" s="42" t="n">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="F74" s="42" t="n">
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="75">
@@ -7168,16 +7168,16 @@
         <v>2939</v>
       </c>
       <c r="C75" s="18" t="n">
-        <v>3256</v>
+        <v>2938</v>
       </c>
       <c r="D75" s="18" t="n">
-        <v>3596</v>
+        <v>3412</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>3480</v>
+        <v>3300</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>3422</v>
+        <v>3244</v>
       </c>
     </row>
     <row r="77">
@@ -7202,16 +7202,16 @@
         <v>-162</v>
       </c>
       <c r="C78" s="27" t="n">
-        <v>-211</v>
+        <v>-200</v>
       </c>
       <c r="D78" s="27" t="n">
-        <v>-206</v>
+        <v>-196</v>
       </c>
       <c r="E78" s="27" t="n">
-        <v>-189</v>
+        <v>-180</v>
       </c>
       <c r="F78" s="27" t="n">
-        <v>-171</v>
+        <v>-163</v>
       </c>
     </row>
     <row r="79">
@@ -7263,16 +7263,16 @@
         <v>-162</v>
       </c>
       <c r="C81" s="18" t="n">
-        <v>-211</v>
+        <v>-200</v>
       </c>
       <c r="D81" s="18" t="n">
-        <v>-206</v>
+        <v>-196</v>
       </c>
       <c r="E81" s="18" t="n">
-        <v>-189</v>
+        <v>-180</v>
       </c>
       <c r="F81" s="18" t="n">
-        <v>-171</v>
+        <v>-163</v>
       </c>
     </row>
     <row r="83">
@@ -7315,16 +7315,16 @@
       </c>
       <c r="B85" s="16" t="n"/>
       <c r="C85" s="27" t="n">
-        <v>-326</v>
+        <v>-310</v>
       </c>
       <c r="D85" s="27" t="n">
-        <v>-1225</v>
+        <v>-1163</v>
       </c>
       <c r="E85" s="27" t="n">
-        <v>-1610</v>
+        <v>-1531</v>
       </c>
       <c r="F85" s="27" t="n">
-        <v>-1643</v>
+        <v>-1563</v>
       </c>
     </row>
     <row r="86">
@@ -7354,16 +7354,16 @@
       </c>
       <c r="B87" s="18" t="n"/>
       <c r="C87" s="18" t="n">
-        <v>-1713</v>
+        <v>-1697</v>
       </c>
       <c r="D87" s="18" t="n">
-        <v>-3588</v>
+        <v>-3526</v>
       </c>
       <c r="E87" s="18" t="n">
-        <v>-4477</v>
+        <v>-4398</v>
       </c>
       <c r="F87" s="18" t="n">
-        <v>-4582</v>
+        <v>-4502</v>
       </c>
     </row>
     <row r="89">
@@ -7374,16 +7374,16 @@
       </c>
       <c r="B89" s="16" t="n"/>
       <c r="C89" s="27" t="n">
-        <v>1332</v>
+        <v>1041</v>
       </c>
       <c r="D89" s="27" t="n">
-        <v>-198</v>
+        <v>-310</v>
       </c>
       <c r="E89" s="27" t="n">
-        <v>-1186</v>
+        <v>-1278</v>
       </c>
       <c r="F89" s="27" t="n">
-        <v>-1331</v>
+        <v>-1421</v>
       </c>
     </row>
     <row r="90">
@@ -7399,13 +7399,13 @@
         <v>1501</v>
       </c>
       <c r="D90" s="27" t="n">
-        <v>2833</v>
+        <v>2542</v>
       </c>
       <c r="E90" s="27" t="n">
-        <v>2636</v>
+        <v>2232</v>
       </c>
       <c r="F90" s="27" t="n">
-        <v>1450</v>
+        <v>954</v>
       </c>
     </row>
     <row r="91">
@@ -7418,16 +7418,16 @@
         <v>1501</v>
       </c>
       <c r="C91" s="18" t="n">
-        <v>2833</v>
+        <v>2542</v>
       </c>
       <c r="D91" s="18" t="n">
-        <v>2636</v>
+        <v>2232</v>
       </c>
       <c r="E91" s="18" t="n">
-        <v>1450</v>
+        <v>954</v>
       </c>
       <c r="F91" s="18" t="n">
-        <v>119</v>
+        <v>-467</v>
       </c>
     </row>
     <row r="93">
@@ -7590,19 +7590,19 @@
         </is>
       </c>
       <c r="B6" s="16" t="n">
-        <v>5929</v>
+        <v>5629</v>
       </c>
       <c r="C6" s="27" t="n">
-        <v>5692</v>
+        <v>5404</v>
       </c>
       <c r="D6" s="27" t="n">
-        <v>5180</v>
+        <v>4917</v>
       </c>
       <c r="E6" s="27" t="n">
-        <v>4662</v>
+        <v>4426</v>
       </c>
       <c r="F6" s="27" t="n">
-        <v>4242</v>
+        <v>4027</v>
       </c>
     </row>
     <row r="7">
@@ -7612,19 +7612,19 @@
         </is>
       </c>
       <c r="B7" s="16" t="n">
-        <v>3011</v>
+        <v>2804</v>
       </c>
       <c r="C7" s="27" t="n">
-        <v>2830</v>
+        <v>2636</v>
       </c>
       <c r="D7" s="27" t="n">
-        <v>2519</v>
+        <v>2346</v>
       </c>
       <c r="E7" s="27" t="n">
-        <v>2217</v>
+        <v>2064</v>
       </c>
       <c r="F7" s="27" t="n">
-        <v>1973</v>
+        <v>1837</v>
       </c>
     </row>
     <row r="8">
@@ -7681,16 +7681,16 @@
         <v>9552</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>9577</v>
+        <v>9095</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>8760</v>
+        <v>8325</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>7935</v>
+        <v>7547</v>
       </c>
       <c r="F10" s="18" t="n">
-        <v>7193</v>
+        <v>6843</v>
       </c>
     </row>
     <row r="11">
@@ -7703,16 +7703,16 @@
         <v>2624</v>
       </c>
       <c r="C11" s="27" t="n">
-        <v>2433</v>
+        <v>2349</v>
       </c>
       <c r="D11" s="27" t="n">
-        <v>2236</v>
+        <v>2161</v>
       </c>
       <c r="E11" s="27" t="n">
-        <v>2041</v>
+        <v>1976</v>
       </c>
       <c r="F11" s="27" t="n">
-        <v>1839</v>
+        <v>1782</v>
       </c>
     </row>
     <row r="12">
@@ -7725,16 +7725,16 @@
         <v>6928</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>7144</v>
+        <v>6746</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>6524</v>
+        <v>6164</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>5894</v>
+        <v>5571</v>
       </c>
       <c r="F12" s="18" t="n">
-        <v>5354</v>
+        <v>5061</v>
       </c>
     </row>
     <row r="13">
@@ -7747,16 +7747,16 @@
         <v>2679</v>
       </c>
       <c r="C13" s="27" t="n">
-        <v>2490</v>
+        <v>2365</v>
       </c>
       <c r="D13" s="27" t="n">
-        <v>2015</v>
+        <v>1915</v>
       </c>
       <c r="E13" s="27" t="n">
-        <v>1587</v>
+        <v>1509</v>
       </c>
       <c r="F13" s="27" t="n">
-        <v>1295</v>
+        <v>1232</v>
       </c>
     </row>
     <row r="14">
@@ -7769,16 +7769,16 @@
         <v>2616</v>
       </c>
       <c r="C14" s="27" t="n">
-        <v>2299</v>
+        <v>2183</v>
       </c>
       <c r="D14" s="27" t="n">
-        <v>1840</v>
+        <v>1748</v>
       </c>
       <c r="E14" s="27" t="n">
-        <v>1428</v>
+        <v>1358</v>
       </c>
       <c r="F14" s="27" t="n">
-        <v>1151</v>
+        <v>1095</v>
       </c>
     </row>
     <row r="15">
@@ -7791,16 +7791,16 @@
         <v>912</v>
       </c>
       <c r="C15" s="27" t="n">
-        <v>862</v>
+        <v>819</v>
       </c>
       <c r="D15" s="27" t="n">
-        <v>701</v>
+        <v>666</v>
       </c>
       <c r="E15" s="27" t="n">
-        <v>595</v>
+        <v>566</v>
       </c>
       <c r="F15" s="27" t="n">
-        <v>504</v>
+        <v>479</v>
       </c>
     </row>
     <row r="16">
@@ -7813,16 +7813,16 @@
         <v>721</v>
       </c>
       <c r="C16" s="18" t="n">
-        <v>1213</v>
+        <v>1114</v>
       </c>
       <c r="D16" s="18" t="n">
-        <v>1712</v>
+        <v>1591</v>
       </c>
       <c r="E16" s="18" t="n">
-        <v>2051</v>
+        <v>1916</v>
       </c>
       <c r="F16" s="18" t="n">
-        <v>2193</v>
+        <v>2054</v>
       </c>
     </row>
     <row r="17">
@@ -7835,16 +7835,16 @@
         <v>0.07548157453936348</v>
       </c>
       <c r="C17" s="25" t="n">
-        <v>0.1266</v>
+        <v>0.1225</v>
       </c>
       <c r="D17" s="25" t="n">
-        <v>0.1955</v>
+        <v>0.1911</v>
       </c>
       <c r="E17" s="25" t="n">
-        <v>0.2585</v>
+        <v>0.2539</v>
       </c>
       <c r="F17" s="25" t="n">
-        <v>0.3049</v>
+        <v>0.3002</v>
       </c>
     </row>
     <row r="18">
@@ -7860,13 +7860,13 @@
         <v>218</v>
       </c>
       <c r="D18" s="26" t="n">
-        <v>290</v>
+        <v>285</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>331</v>
+        <v>322</v>
       </c>
       <c r="F18" s="26" t="n">
-        <v>351</v>
+        <v>339</v>
       </c>
     </row>
     <row r="19">
@@ -7901,16 +7901,16 @@
         <v>1009</v>
       </c>
       <c r="C20" s="27" t="n">
-        <v>1326</v>
+        <v>1227</v>
       </c>
       <c r="D20" s="27" t="n">
-        <v>1898</v>
+        <v>1771</v>
       </c>
       <c r="E20" s="27" t="n">
-        <v>2278</v>
+        <v>2133</v>
       </c>
       <c r="F20" s="27" t="n">
-        <v>2440</v>
+        <v>2289</v>
       </c>
     </row>
     <row r="21">
@@ -7923,16 +7923,16 @@
         <v>-316</v>
       </c>
       <c r="C21" s="27" t="n">
-        <v>-331</v>
+        <v>-307</v>
       </c>
       <c r="D21" s="27" t="n">
-        <v>-475</v>
+        <v>-443</v>
       </c>
       <c r="E21" s="27" t="n">
-        <v>-569</v>
+        <v>-533</v>
       </c>
       <c r="F21" s="27" t="n">
-        <v>-610</v>
+        <v>-572</v>
       </c>
     </row>
     <row r="22">
@@ -7945,16 +7945,16 @@
         <v>693</v>
       </c>
       <c r="C22" s="18" t="n">
-        <v>994</v>
+        <v>920</v>
       </c>
       <c r="D22" s="18" t="n">
-        <v>1424</v>
+        <v>1329</v>
       </c>
       <c r="E22" s="18" t="n">
-        <v>1708</v>
+        <v>1600</v>
       </c>
       <c r="F22" s="18" t="n">
-        <v>1830</v>
+        <v>1717</v>
       </c>
     </row>
     <row r="23">
@@ -7989,16 +7989,16 @@
         <v>2.59</v>
       </c>
       <c r="C24" s="32" t="n">
-        <v>3.81</v>
+        <v>3.52</v>
       </c>
       <c r="D24" s="32" t="n">
-        <v>5.65</v>
+        <v>5.27</v>
       </c>
       <c r="E24" s="32" t="n">
-        <v>7.06</v>
+        <v>6.61</v>
       </c>
       <c r="F24" s="32" t="n">
-        <v>7.88</v>
+        <v>7.39</v>
       </c>
     </row>
     <row r="26">
@@ -8035,16 +8035,16 @@
         <v>1501</v>
       </c>
       <c r="C28" s="27" t="n">
-        <v>2975</v>
+        <v>2704</v>
       </c>
       <c r="D28" s="27" t="n">
-        <v>4125</v>
+        <v>3742</v>
       </c>
       <c r="E28" s="27" t="n">
-        <v>5137</v>
+        <v>4649</v>
       </c>
       <c r="F28" s="27" t="n">
-        <v>6347</v>
+        <v>5754</v>
       </c>
     </row>
     <row r="29">
@@ -8079,16 +8079,16 @@
         <v>2332</v>
       </c>
       <c r="C30" s="27" t="n">
-        <v>2338</v>
+        <v>2220</v>
       </c>
       <c r="D30" s="27" t="n">
-        <v>2139</v>
+        <v>2032</v>
       </c>
       <c r="E30" s="27" t="n">
-        <v>1937</v>
+        <v>1843</v>
       </c>
       <c r="F30" s="27" t="n">
-        <v>1756</v>
+        <v>1671</v>
       </c>
     </row>
     <row r="31">
@@ -8101,16 +8101,16 @@
         <v>348</v>
       </c>
       <c r="C31" s="27" t="n">
-        <v>345</v>
+        <v>327</v>
       </c>
       <c r="D31" s="27" t="n">
-        <v>315</v>
+        <v>300</v>
       </c>
       <c r="E31" s="27" t="n">
-        <v>286</v>
+        <v>272</v>
       </c>
       <c r="F31" s="27" t="n">
-        <v>259</v>
+        <v>246</v>
       </c>
     </row>
     <row r="32">
@@ -8123,16 +8123,16 @@
         <v>306</v>
       </c>
       <c r="C32" s="27" t="n">
-        <v>306</v>
+        <v>291</v>
       </c>
       <c r="D32" s="27" t="n">
-        <v>280</v>
+        <v>266</v>
       </c>
       <c r="E32" s="27" t="n">
-        <v>254</v>
+        <v>242</v>
       </c>
       <c r="F32" s="27" t="n">
-        <v>230</v>
+        <v>219</v>
       </c>
     </row>
     <row r="33">
@@ -8145,16 +8145,16 @@
         <v>1093</v>
       </c>
       <c r="C33" s="27" t="n">
-        <v>1048</v>
+        <v>1038</v>
       </c>
       <c r="D33" s="27" t="n">
-        <v>971</v>
+        <v>952</v>
       </c>
       <c r="E33" s="27" t="n">
-        <v>863</v>
+        <v>836</v>
       </c>
       <c r="F33" s="27" t="n">
-        <v>725</v>
+        <v>691</v>
       </c>
     </row>
     <row r="34">
@@ -8233,16 +8233,16 @@
         <v>634</v>
       </c>
       <c r="C37" s="27" t="n">
-        <v>632</v>
+        <v>600</v>
       </c>
       <c r="D37" s="27" t="n">
-        <v>578</v>
+        <v>549</v>
       </c>
       <c r="E37" s="27" t="n">
-        <v>524</v>
+        <v>498</v>
       </c>
       <c r="F37" s="27" t="n">
-        <v>475</v>
+        <v>452</v>
       </c>
     </row>
     <row r="38">
@@ -8299,16 +8299,16 @@
         <v>18074</v>
       </c>
       <c r="C40" s="18" t="n">
-        <v>19405</v>
+        <v>18942</v>
       </c>
       <c r="D40" s="18" t="n">
-        <v>20069</v>
+        <v>19502</v>
       </c>
       <c r="E40" s="18" t="n">
-        <v>20561</v>
+        <v>19899</v>
       </c>
       <c r="F40" s="18" t="n">
-        <v>21252</v>
+        <v>20492</v>
       </c>
     </row>
     <row r="42">
@@ -8333,16 +8333,16 @@
         <v>142</v>
       </c>
       <c r="C43" s="27" t="n">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="D43" s="27" t="n">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E43" s="27" t="n">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="F43" s="27" t="n">
-        <v>108</v>
+        <v>103</v>
       </c>
     </row>
     <row r="44">
@@ -8355,16 +8355,16 @@
         <v>642</v>
       </c>
       <c r="C44" s="27" t="n">
-        <v>651</v>
+        <v>618</v>
       </c>
       <c r="D44" s="27" t="n">
-        <v>596</v>
+        <v>566</v>
       </c>
       <c r="E44" s="27" t="n">
-        <v>540</v>
+        <v>513</v>
       </c>
       <c r="F44" s="27" t="n">
-        <v>489</v>
+        <v>465</v>
       </c>
     </row>
     <row r="45">
@@ -8377,16 +8377,16 @@
         <v>454</v>
       </c>
       <c r="C45" s="27" t="n">
-        <v>460</v>
+        <v>437</v>
       </c>
       <c r="D45" s="27" t="n">
-        <v>420</v>
+        <v>400</v>
       </c>
       <c r="E45" s="27" t="n">
-        <v>381</v>
+        <v>362</v>
       </c>
       <c r="F45" s="27" t="n">
-        <v>345</v>
+        <v>328</v>
       </c>
     </row>
     <row r="46">
@@ -8399,16 +8399,16 @@
         <v>5010</v>
       </c>
       <c r="C46" s="27" t="n">
-        <v>4760</v>
+        <v>4507</v>
       </c>
       <c r="D46" s="27" t="n">
-        <v>4399</v>
+        <v>4170</v>
       </c>
       <c r="E46" s="27" t="n">
-        <v>3974</v>
+        <v>3770</v>
       </c>
       <c r="F46" s="27" t="n">
-        <v>3603</v>
+        <v>3419</v>
       </c>
     </row>
     <row r="47">
@@ -8531,16 +8531,16 @@
         <v>10269</v>
       </c>
       <c r="C52" s="18" t="n">
-        <v>10036</v>
+        <v>9720</v>
       </c>
       <c r="D52" s="18" t="n">
-        <v>9568</v>
+        <v>9282</v>
       </c>
       <c r="E52" s="18" t="n">
-        <v>9035</v>
+        <v>8780</v>
       </c>
       <c r="F52" s="18" t="n">
-        <v>8566</v>
+        <v>8336</v>
       </c>
     </row>
     <row r="54">
@@ -8565,16 +8565,16 @@
         <v>12673</v>
       </c>
       <c r="C55" s="27" t="n">
-        <v>14110</v>
+        <v>14037</v>
       </c>
       <c r="D55" s="27" t="n">
-        <v>15249</v>
+        <v>15119</v>
       </c>
       <c r="E55" s="27" t="n">
-        <v>16122</v>
+        <v>15949</v>
       </c>
       <c r="F55" s="27" t="n">
-        <v>16841</v>
+        <v>16633</v>
       </c>
     </row>
     <row r="56">
@@ -8609,16 +8609,16 @@
         <v>-512</v>
       </c>
       <c r="C57" s="27" t="n">
-        <v>482</v>
+        <v>408</v>
       </c>
       <c r="D57" s="27" t="n">
-        <v>1538</v>
+        <v>1387</v>
       </c>
       <c r="E57" s="27" t="n">
-        <v>2730</v>
+        <v>2496</v>
       </c>
       <c r="F57" s="27" t="n">
-        <v>4042</v>
+        <v>3720</v>
       </c>
     </row>
     <row r="58">
@@ -8653,16 +8653,16 @@
         <v>7805</v>
       </c>
       <c r="C59" s="18" t="n">
-        <v>9369</v>
+        <v>9222</v>
       </c>
       <c r="D59" s="18" t="n">
-        <v>10501</v>
+        <v>10220</v>
       </c>
       <c r="E59" s="18" t="n">
-        <v>11526</v>
+        <v>11119</v>
       </c>
       <c r="F59" s="18" t="n">
-        <v>12686</v>
+        <v>12156</v>
       </c>
     </row>
     <row r="61">
@@ -8721,16 +8721,16 @@
         <v>693</v>
       </c>
       <c r="C65" s="27" t="n">
-        <v>994</v>
+        <v>920</v>
       </c>
       <c r="D65" s="27" t="n">
-        <v>1424</v>
+        <v>1329</v>
       </c>
       <c r="E65" s="27" t="n">
-        <v>1708</v>
+        <v>1600</v>
       </c>
       <c r="F65" s="27" t="n">
-        <v>1830</v>
+        <v>1717</v>
       </c>
     </row>
     <row r="66">
@@ -8787,16 +8787,16 @@
         <v>1626</v>
       </c>
       <c r="C68" s="27" t="n">
-        <v>1437</v>
+        <v>1364</v>
       </c>
       <c r="D68" s="27" t="n">
-        <v>1139</v>
+        <v>1082</v>
       </c>
       <c r="E68" s="27" t="n">
-        <v>873</v>
+        <v>830</v>
       </c>
       <c r="F68" s="27" t="n">
-        <v>719</v>
+        <v>684</v>
       </c>
     </row>
     <row r="69">
@@ -8807,16 +8807,16 @@
       </c>
       <c r="B69" s="40" t="n"/>
       <c r="C69" s="42" t="n">
-        <v>-6</v>
+        <v>112</v>
       </c>
       <c r="D69" s="42" t="n">
-        <v>199</v>
+        <v>188</v>
       </c>
       <c r="E69" s="42" t="n">
-        <v>201</v>
+        <v>190</v>
       </c>
       <c r="F69" s="42" t="n">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="70">
@@ -8827,16 +8827,16 @@
       </c>
       <c r="B70" s="40" t="n"/>
       <c r="C70" s="42" t="n">
-        <v>-250</v>
+        <v>-503</v>
       </c>
       <c r="D70" s="42" t="n">
-        <v>-361</v>
+        <v>-337</v>
       </c>
       <c r="E70" s="42" t="n">
-        <v>-425</v>
+        <v>-400</v>
       </c>
       <c r="F70" s="42" t="n">
-        <v>-372</v>
+        <v>-352</v>
       </c>
     </row>
     <row r="71">
@@ -8847,16 +8847,16 @@
       </c>
       <c r="B71" s="40" t="n"/>
       <c r="C71" s="42" t="n">
-        <v>9</v>
+        <v>-24</v>
       </c>
       <c r="D71" s="42" t="n">
-        <v>-56</v>
+        <v>-52</v>
       </c>
       <c r="E71" s="42" t="n">
-        <v>-56</v>
+        <v>-53</v>
       </c>
       <c r="F71" s="42" t="n">
-        <v>-50</v>
+        <v>-48</v>
       </c>
     </row>
     <row r="72">
@@ -8867,16 +8867,16 @@
       </c>
       <c r="B72" s="40" t="n"/>
       <c r="C72" s="42" t="n">
-        <v>7</v>
+        <v>-23</v>
       </c>
       <c r="D72" s="42" t="n">
-        <v>-51</v>
+        <v>-49</v>
       </c>
       <c r="E72" s="42" t="n">
-        <v>-52</v>
+        <v>-49</v>
       </c>
       <c r="F72" s="42" t="n">
-        <v>-47</v>
+        <v>-44</v>
       </c>
     </row>
     <row r="73">
@@ -8887,16 +8887,16 @@
       </c>
       <c r="B73" s="40" t="n"/>
       <c r="C73" s="42" t="n">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="D73" s="42" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E73" s="42" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="F73" s="42" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="74">
@@ -8907,16 +8907,16 @@
       </c>
       <c r="B74" s="40" t="n"/>
       <c r="C74" s="42" t="n">
-        <v>1</v>
+        <v>49</v>
       </c>
       <c r="D74" s="42" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="E74" s="42" t="n">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="F74" s="42" t="n">
-        <v>73</v>
+        <v>69</v>
       </c>
     </row>
     <row r="75">
@@ -8928,16 +8928,16 @@
         <v>2939</v>
       </c>
       <c r="C75" s="18" t="n">
-        <v>2533</v>
+        <v>2252</v>
       </c>
       <c r="D75" s="18" t="n">
-        <v>2756</v>
+        <v>2616</v>
       </c>
       <c r="E75" s="18" t="n">
-        <v>2727</v>
+        <v>2589</v>
       </c>
       <c r="F75" s="18" t="n">
-        <v>2743</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="77">
@@ -8962,16 +8962,16 @@
         <v>-162</v>
       </c>
       <c r="C78" s="27" t="n">
-        <v>-192</v>
+        <v>-182</v>
       </c>
       <c r="D78" s="27" t="n">
-        <v>-175</v>
+        <v>-166</v>
       </c>
       <c r="E78" s="27" t="n">
-        <v>-159</v>
+        <v>-151</v>
       </c>
       <c r="F78" s="27" t="n">
-        <v>-144</v>
+        <v>-137</v>
       </c>
     </row>
     <row r="79">
@@ -9023,16 +9023,16 @@
         <v>-162</v>
       </c>
       <c r="C81" s="18" t="n">
-        <v>-192</v>
+        <v>-182</v>
       </c>
       <c r="D81" s="18" t="n">
-        <v>-175</v>
+        <v>-166</v>
       </c>
       <c r="E81" s="18" t="n">
-        <v>-159</v>
+        <v>-151</v>
       </c>
       <c r="F81" s="18" t="n">
-        <v>-144</v>
+        <v>-137</v>
       </c>
     </row>
     <row r="83">
@@ -9078,13 +9078,13 @@
         <v>-0</v>
       </c>
       <c r="D85" s="27" t="n">
-        <v>-368</v>
+        <v>-350</v>
       </c>
       <c r="E85" s="27" t="n">
-        <v>-516</v>
+        <v>-491</v>
       </c>
       <c r="F85" s="27" t="n">
-        <v>-518</v>
+        <v>-493</v>
       </c>
     </row>
     <row r="86">
@@ -9117,13 +9117,13 @@
         <v>-867</v>
       </c>
       <c r="D87" s="18" t="n">
-        <v>-1431</v>
+        <v>-1413</v>
       </c>
       <c r="E87" s="18" t="n">
-        <v>-1556</v>
+        <v>-1531</v>
       </c>
       <c r="F87" s="18" t="n">
-        <v>-1389</v>
+        <v>-1364</v>
       </c>
     </row>
     <row r="89">
@@ -9134,16 +9134,16 @@
       </c>
       <c r="B89" s="16" t="n"/>
       <c r="C89" s="27" t="n">
-        <v>1474</v>
+        <v>1203</v>
       </c>
       <c r="D89" s="27" t="n">
-        <v>1150</v>
+        <v>1037</v>
       </c>
       <c r="E89" s="27" t="n">
-        <v>1012</v>
+        <v>907</v>
       </c>
       <c r="F89" s="27" t="n">
-        <v>1210</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="90">
@@ -9159,13 +9159,13 @@
         <v>1501</v>
       </c>
       <c r="D90" s="27" t="n">
-        <v>2975</v>
+        <v>2704</v>
       </c>
       <c r="E90" s="27" t="n">
-        <v>4125</v>
+        <v>3742</v>
       </c>
       <c r="F90" s="27" t="n">
-        <v>5137</v>
+        <v>4649</v>
       </c>
     </row>
     <row r="91">
@@ -9178,16 +9178,16 @@
         <v>1501</v>
       </c>
       <c r="C91" s="18" t="n">
-        <v>2975</v>
+        <v>2704</v>
       </c>
       <c r="D91" s="18" t="n">
-        <v>4125</v>
+        <v>3742</v>
       </c>
       <c r="E91" s="18" t="n">
-        <v>5137</v>
+        <v>4649</v>
       </c>
       <c r="F91" s="18" t="n">
-        <v>6347</v>
+        <v>5754</v>
       </c>
     </row>
     <row r="93">
@@ -9391,16 +9391,16 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.2067</v>
+        <v>0.1454</v>
       </c>
       <c r="D11" s="10" t="n">
-        <v>0.1752</v>
+        <v>0.1769</v>
       </c>
       <c r="E11" s="10" t="n">
-        <v>0.1817</v>
+        <v>0.184</v>
       </c>
       <c r="F11" s="10" t="n">
-        <v>0.1606</v>
+        <v>0.1625</v>
       </c>
     </row>
     <row r="12">
@@ -9415,16 +9415,16 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>0.1024</v>
+        <v>0.0465</v>
       </c>
       <c r="D12" s="10" t="n">
-        <v>-0.0227</v>
+        <v>-0.0219</v>
       </c>
       <c r="E12" s="10" t="n">
-        <v>-0.07969999999999999</v>
+        <v>-0.0789</v>
       </c>
       <c r="F12" s="10" t="n">
-        <v>-0.0964</v>
+        <v>-0.09619999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -9439,16 +9439,16 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>0.0026</v>
+        <v>-0.0478</v>
       </c>
       <c r="D13" s="10" t="n">
-        <v>-0.0853</v>
+        <v>-0.0847</v>
       </c>
       <c r="E13" s="10" t="n">
-        <v>-0.09420000000000001</v>
+        <v>-0.0935</v>
       </c>
       <c r="F13" s="10" t="n">
-        <v>-0.0935</v>
+        <v>-0.09329999999999999</v>
       </c>
     </row>
     <row r="15">
@@ -9535,16 +9535,16 @@
         </is>
       </c>
       <c r="C19" s="10" t="n">
-        <v>0.2473</v>
+        <v>0.2511</v>
       </c>
       <c r="D19" s="10" t="n">
-        <v>0.2428</v>
+        <v>0.2464</v>
       </c>
       <c r="E19" s="10" t="n">
-        <v>0.2374</v>
+        <v>0.2408</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>0.2284</v>
+        <v>0.2315</v>
       </c>
     </row>
     <row r="20">
@@ -9559,16 +9559,16 @@
         </is>
       </c>
       <c r="C20" s="10" t="n">
-        <v>0.2496</v>
+        <v>0.2535</v>
       </c>
       <c r="D20" s="10" t="n">
-        <v>0.2484</v>
+        <v>0.2524</v>
       </c>
       <c r="E20" s="10" t="n">
-        <v>0.2493</v>
+        <v>0.2535</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>0.2482</v>
+        <v>0.2525</v>
       </c>
     </row>
     <row r="21">
@@ -9583,16 +9583,16 @@
         </is>
       </c>
       <c r="C21" s="10" t="n">
-        <v>0.2541</v>
+        <v>0.2582</v>
       </c>
       <c r="D21" s="10" t="n">
-        <v>0.2552</v>
+        <v>0.2596</v>
       </c>
       <c r="E21" s="10" t="n">
-        <v>0.2572</v>
+        <v>0.2618</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>0.2558</v>
+        <v>0.2605</v>
       </c>
     </row>
     <row r="23">
@@ -9640,7 +9640,7 @@
         <v>0.16</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>0.1301</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="25">
@@ -9661,7 +9661,7 @@
         <v>0.23</v>
       </c>
       <c r="E25" s="10" t="n">
-        <v>0.2</v>
+        <v>0.1999</v>
       </c>
       <c r="F25" s="10" t="n">
         <v>0.18</v>
@@ -9727,13 +9727,13 @@
         </is>
       </c>
       <c r="C29" s="10" t="n">
-        <v>0.2401</v>
+        <v>0.24</v>
       </c>
       <c r="D29" s="10" t="n">
         <v>0.21</v>
       </c>
       <c r="E29" s="10" t="n">
-        <v>0.18</v>
+        <v>0.1799</v>
       </c>
       <c r="F29" s="10" t="n">
         <v>0.16</v>
@@ -9808,7 +9808,7 @@
         <v>0.075</v>
       </c>
       <c r="F33" s="10" t="n">
-        <v>0.0701</v>
+        <v>0.07000000000000001</v>
       </c>
     </row>
     <row r="35">
@@ -9847,7 +9847,7 @@
         </is>
       </c>
       <c r="C36" s="10" t="n">
-        <v>0.13</v>
+        <v>0.1301</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>0.09</v>
@@ -9943,10 +9943,10 @@
         </is>
       </c>
       <c r="C41" s="10" t="n">
-        <v>0.3</v>
+        <v>0.2999</v>
       </c>
       <c r="D41" s="10" t="n">
-        <v>0.3</v>
+        <v>0.2999</v>
       </c>
       <c r="E41" s="10" t="n">
         <v>0.28</v>
@@ -14686,7 +14686,7 @@
         <v/>
       </c>
       <c r="C4" s="8" t="n">
-        <v>740.9299999999999</v>
+        <v>722.85</v>
       </c>
       <c r="D4" s="10">
         <f>C4/129.34-1</f>
@@ -14712,7 +14712,7 @@
         <v/>
       </c>
       <c r="C5" s="8" t="n">
-        <v>128.2</v>
+        <v>125.12</v>
       </c>
       <c r="D5" s="10">
         <f>C5/129.34-1</f>
@@ -14738,7 +14738,7 @@
         <v/>
       </c>
       <c r="C6" s="8" t="n">
-        <v>69.81</v>
+        <v>68.55</v>
       </c>
       <c r="D6" s="10">
         <f>C6/129.34-1</f>
@@ -15148,7 +15148,7 @@
         <v>129.34</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>605.53</v>
+        <v>590.6900000000001</v>
       </c>
       <c r="F5" s="7">
         <f>E5-D5</f>
@@ -15183,7 +15183,7 @@
         <v/>
       </c>
       <c r="O5" s="10" t="n">
-        <v>0.6729999999999999</v>
+        <v>0.659</v>
       </c>
       <c r="P5" s="30" t="n">
         <v>268</v>
@@ -15210,7 +15210,7 @@
         <v>129.34</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>740.9299999999999</v>
+        <v>722.85</v>
       </c>
       <c r="F6" s="7">
         <f>E6-D6</f>
@@ -15245,7 +15245,7 @@
         <v/>
       </c>
       <c r="O6" s="10" t="n">
-        <v>0.547</v>
+        <v>0.5379999999999999</v>
       </c>
       <c r="P6" s="30" t="n">
         <v>268</v>
@@ -15272,14 +15272,14 @@
         <v>129.34</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>129.83</v>
+        <v>126.56</v>
       </c>
       <c r="F7" s="7">
         <f>E7-D7</f>
         <v/>
       </c>
       <c r="G7" s="6" t="n">
-        <v>12.71</v>
+        <v>12.08</v>
       </c>
       <c r="H7" s="8" t="n">
         <v>6617</v>
@@ -15307,7 +15307,7 @@
         <v/>
       </c>
       <c r="O7" s="10" t="n">
-        <v>0.033</v>
+        <v>0.023</v>
       </c>
       <c r="P7" s="30" t="n">
         <v>268</v>
@@ -15334,14 +15334,14 @@
         <v>129.34</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>128.2</v>
+        <v>125.12</v>
       </c>
       <c r="F8" s="7">
         <f>E8-D8</f>
         <v/>
       </c>
       <c r="G8" s="6" t="n">
-        <v>20.26</v>
+        <v>19.26</v>
       </c>
       <c r="H8" s="8" t="n">
         <v>9556</v>
@@ -15369,7 +15369,7 @@
         <v/>
       </c>
       <c r="O8" s="10" t="n">
-        <v>0.035</v>
+        <v>0.028</v>
       </c>
       <c r="P8" s="30" t="n">
         <v>268</v>
@@ -15396,14 +15396,14 @@
         <v>129.34</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>75.38</v>
+        <v>73.92</v>
       </c>
       <c r="F9" s="7">
         <f>E9-D9</f>
         <v/>
       </c>
       <c r="G9" s="6" t="n">
-        <v>3.46</v>
+        <v>3.29</v>
       </c>
       <c r="H9" s="8" t="n">
         <v>2970</v>
@@ -15431,7 +15431,7 @@
         <v/>
       </c>
       <c r="O9" s="10" t="n">
-        <v>-0.152</v>
+        <v>-0.158</v>
       </c>
       <c r="P9" s="30" t="n">
         <v>268</v>
@@ -15458,14 +15458,14 @@
         <v>129.34</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>69.81</v>
+        <v>68.55</v>
       </c>
       <c r="F10" s="7">
         <f>E10-D10</f>
         <v/>
       </c>
       <c r="G10" s="6" t="n">
-        <v>5.6</v>
+        <v>5.33</v>
       </c>
       <c r="H10" s="8" t="n">
         <v>3841</v>
@@ -15493,7 +15493,7 @@
         <v/>
       </c>
       <c r="O10" s="10" t="n">
-        <v>-0.126</v>
+        <v>-0.131</v>
       </c>
       <c r="P10" s="30" t="n">
         <v>268</v>
@@ -15509,7 +15509,7 @@
         </is>
       </c>
       <c r="M12" s="9" t="n">
-        <v>1.207</v>
+        <v>1.153</v>
       </c>
     </row>
     <row r="13">
@@ -15519,7 +15519,7 @@
         </is>
       </c>
       <c r="M13" s="9" t="n">
-        <v>1.582</v>
+        <v>1.518</v>
       </c>
     </row>
     <row r="15">

</xml_diff>